<commit_message>
Update AeroSense wiki without CTB files
</commit_message>
<xml_diff>
--- a/hardware information/AeroSense v2/05_BOM/BOM_ZH.xlsx
+++ b/hardware information/AeroSense v2/05_BOM/BOM_ZH.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R671d611e21444852"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Printed" sheetId="2" r:id="Rddd6d65d73524979"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase" sheetId="3" r:id="Ree3fb7a64ef44e72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCB" sheetId="4" r:id="Rbd6284f90c5a4e0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print_batches" sheetId="5" r:id="Re06c295592a2429c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re37e9c86e15f4b48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Printed" sheetId="2" r:id="Rdd33a48358a34474"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase" sheetId="3" r:id="R23daecd220b64d0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCB" sheetId="4" r:id="R4f7b0463448249b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print_batches" sheetId="5" r:id="Rd7041de6576e4d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="6" r:id="R6ea0f7d293a741aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +21,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="#,##0.00;(#,##0.00);0.00"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -53,8 +54,20 @@
       <x:color rgb="FF243746"/>
       <x:name val="Microsoft JhengHei"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF263D50"/>
+      <x:name val="Microsoft JhengHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF263D50"/>
+      <x:name val="Microsoft JhengHei"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -71,6 +84,16 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF263D50"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDFE8EE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -78,7 +101,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -124,6 +147,33 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -12623,7 +12673,7 @@
       </x:c>
       <x:c r="C14" s="2"/>
       <x:c r="D14" s="2" t="str">
-        <x:v>P2 與 P3 合印；不虛構個別零件單價。cost.md 原檔不變。</x:v>
+        <x:v>P2 與 P3 合印，不虛構個別零件單價。原始成本及差異已保存於 Notes。</x:v>
       </x:c>
       <x:c r="E14" s="2"/>
       <x:c r="F14" s="2"/>
@@ -14125,4 +14175,3176 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF7B8991"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="105" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="90" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="18"/>
+      <x:c r="B1" s="18"/>
+      <x:c r="C1" s="18"/>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="19" t="str">
+        <x:v>說明與來源</x:v>
+      </x:c>
+      <x:c r="B2" s="18" t="str">
+        <x:v>2026-10-11 整併。原有預算輸入與公式保留。</x:v>
+      </x:c>
+      <x:c r="C2" s="18"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="18"/>
+      <x:c r="B3" s="18"/>
+      <x:c r="C3" s="18"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="22" t="str">
+        <x:v>主題／識別</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>說明／保留的來源明細</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>來源／備查</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="25" t="str">
+        <x:v>工作簿使用說明</x:v>
+      </x:c>
+      <x:c r="B5" s="25" t="str"/>
+      <x:c r="C5" s="25" t="str"/>
+    </x:row>
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="A6" s="18" t="str">
+        <x:v>完整 BOM</x:v>
+      </x:c>
+      <x:c r="B6" s="18" t="str">
+        <x:v>原有五張工作表包含 8 個列印件、26 列採購項、61 列 PCB 及 3 個列印批次。Summary 保留可重算的預算公式。</x:v>
+      </x:c>
+      <x:c r="C6" s="18" t="str"/>
+    </x:row>
+    <x:row r="7" ht="28" customHeight="1">
+      <x:c r="A7" s="18" t="str">
+        <x:v>幣別與更新</x:v>
+      </x:c>
+      <x:c r="B7" s="18" t="str">
+        <x:v>中文工作簿維持 NTD 與 USD。價格來源保留原幣別。Summary 的匯率輸入控制現有換算公式。</x:v>
+      </x:c>
+      <x:c r="C7" s="18" t="str"/>
+    </x:row>
+    <x:row r="8" ht="40" customHeight="1">
+      <x:c r="A8" s="18" t="str">
+        <x:v>預算說明 1</x:v>
+      </x:c>
+      <x:c r="B8" s="18" t="str">
+        <x:v>2026-10-08。工作簿同時列出 NTD 與 USD。分類改為「必要、開發者購買、未來展望」，並保留 STL、PCB、外購材料三種明細。價格來源、實際用途與待確認規格分開列。</x:v>
+      </x:c>
+      <x:c r="C8" s="18" t="str">
+        <x:v>原預算讀法；來源價格日期為 2026-10-08。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="40" customHeight="1">
+      <x:c r="A9" s="18" t="str">
+        <x:v>預算說明 2</x:v>
+      </x:c>
+      <x:c r="B9" s="18" t="str">
+        <x:v>必要：八件列印件、PCB 及 13 列外購裝配材料。開發者購買：10 列機外燒錄、量測、給氣與工具；可以借用，但給氣與流量確認能力仍是實驗必要條件。未來展望：PDMS 膜、氣閥驅動、環境感測共三列，不加進當前機器預算。</x:v>
+      </x:c>
+      <x:c r="C9" s="18" t="str">
+        <x:v>原預算讀法；來源價格日期為 2026-10-08。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="54" customHeight="1">
+      <x:c r="A10" s="18" t="str">
+        <x:v>預算說明 3</x:v>
+      </x:c>
+      <x:c r="B10" s="18" t="str">
+        <x:v> 上述是預算，不是已確認可下單總價。 單機包含 NTD 12,000 客製薄型螢光濾片預留；參考的 Edmund 67-016 價格 USD 284，但其 12.5 mm 外徑與約 2 mm 厚度均不符合現有 5.2 × 4.2 × 1.0 mm 濾片座。不能直接購買並假設可裝，也不能只裁切外形就解決厚度問題。尚需尺寸、角度光譜與加工報價。</x:v>
+      </x:c>
+      <x:c r="C10" s="18" t="str">
+        <x:v>原預算讀法；來源價格日期為 2026-10-08。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="40" customHeight="1">
+      <x:c r="A11" s="18" t="str">
+        <x:v>預算說明 4</x:v>
+      </x:c>
+      <x:c r="B11" s="18" t="str">
+        <x:v>四組光學報告另比較 Edmund #29-190、500 nm 超薄 OD4 候選，與舊預算參考 #67-016 不同。情境光譜及 12.45 mm 圓片尺寸不代表已能裝入現有濾片座。選定濾片與固定座並取得確認報價前，仍保留原客製濾片預算。</x:v>
+      </x:c>
+      <x:c r="C11" s="18" t="str">
+        <x:v>原預算讀法；來源價格日期為 2026-10-08。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="40" customHeight="1">
+      <x:c r="A12" s="18" t="str">
+        <x:v>預算說明 5</x:v>
+      </x:c>
+      <x:c r="B12" s="18" t="str">
+        <x:v>Listed＝可查到商品價；Proxy＝類似品或包裝差異的參考；Allowance／Custom allowance＝工程預留額。沒有公開且相符的價格時，不把預留額寫成已查核市價。螺絲長度、M3 標準螺帽及墊片規格不因價格參考品而更換。</x:v>
+      </x:c>
+      <x:c r="C12" s="18" t="str">
+        <x:v>原預算讀法；來源價格日期為 2026-10-08。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="54" customHeight="1">
+      <x:c r="A13" s="18" t="str">
+        <x:v>預算說明 6</x:v>
+      </x:c>
+      <x:c r="B13" s="18" t="str">
+        <x:v>濾器參考品為 Gilson ANP1322，USD 95／100 個；兩個用量換算 NTD 60.43，但買一盒是 NTD 3,021.48。它是 0.22 µm、非無菌疏水 PTFE 參考品，不代表已符合原設計 0.2 µm 氣體濾器要求。細胞用途、接頭、壓降與 VOC 回收仍需確認。</x:v>
+      </x:c>
+      <x:c r="C13" s="18" t="str">
+        <x:v>原預算讀法；來源價格日期為 2026-10-08。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="40" customHeight="1">
+      <x:c r="A14" s="18" t="str">
+        <x:v>預算說明 7</x:v>
+      </x:c>
+      <x:c r="B14" s="18" t="str">
+        <x:v>已持有量 K 欄預設 0。填入已買或可借數量，需購包數 P 與新購額 Q/R 會重算；用量成本 N/O 不會因此歸零。預留額不是採購授權，也不代表必須購買新的實驗室儀器。</x:v>
+      </x:c>
+      <x:c r="C14" s="18" t="str">
+        <x:v>原預算讀法；來源價格日期為 2026-10-08。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="54" customHeight="1">
+      <x:c r="A15" s="18" t="str">
+        <x:v>預算說明 8</x:v>
+      </x:c>
+      <x:c r="B15" s="18" t="str">
+        <x:v>PCB 保留 61 列原始位號、數量與數值。已列零件材料估價為 NTD 1,954.00；U3 身分未知，留白。許多被動元件尚缺值或封裝，僅列通用預算，不能據此採購。FD 光學點與 H 固定孔為製板特徵，材料单價 0 不是漏列。PCB 零件估價不另加到 NT$131,250／2 片的含設計與開機報價。</x:v>
+      </x:c>
+      <x:c r="C15" s="18" t="str">
+        <x:v>原預算讀法；來源價格日期為 2026-10-08。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="40" customHeight="1">
+      <x:c r="A16" s="18" t="str">
+        <x:v>預算說明 9</x:v>
+      </x:c>
+      <x:c r="B16" s="18" t="str">
+        <x:v>列印維持 1.2 × (25 + 原樹脂小計 × 1.1 + 分鐘/60 × 7.195)。三批分別 525.31282、535.12550、54.94728 NTD；全精度相加 1115.38560。合印批次不假造單件價格。原始列印筆記已保存於下方。</x:v>
+      </x:c>
+      <x:c r="C16" s="18" t="str">
+        <x:v>原預算讀法；來源價格日期為 2026-10-08。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="40" customHeight="1">
+      <x:c r="A17" s="18" t="str">
+        <x:v>預算說明 10</x:v>
+      </x:c>
+      <x:c r="B17" s="18" t="str">
+        <x:v>匯率採臺灣銀行頁面顯示的 2026-10-05 15:13 美元即期賣出 31.805 NTD/USD；2026-10-08 查閱。這是比較用快照，不是 10 月 8 日成交匯率。USD 價來源保持 USD 輸入，NTD 價保持 NTD 輸入，改匯率會正確換算兩者。</x:v>
+      </x:c>
+      <x:c r="C17" s="18" t="str">
+        <x:v>原預算讀法；來源價格日期為 2026-10-08。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="40" customHeight="1">
+      <x:c r="A18" s="18" t="str">
+        <x:v>預算說明 11</x:v>
+      </x:c>
+      <x:c r="B18" s="18" t="str">
+        <x:v>未含運費、額外稅金、未列人工、失敗重印、細胞培養耗材及既有印表機、後固化機、手機、電腦、培養設施的重購成本。</x:v>
+      </x:c>
+      <x:c r="C18" s="18" t="str">
+        <x:v>原預算讀法；來源價格日期為 2026-10-08。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="25" t="str">
+        <x:v>原始列印成本紀錄</x:v>
+      </x:c>
+      <x:c r="B19" s="25" t="str"/>
+      <x:c r="C19" s="25" t="str"/>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="A20" s="18" t="str">
+        <x:v>印表機與切片批次</x:v>
+      </x:c>
+      <x:c r="B20" s="18" t="str">
+        <x:v>Phrozen Sonic Mighty Revo 16K. P1: 01_base_BLACK.ctb; P2: 020308_parts.ctb; P3: 0407_wells.ctb.</x:v>
+      </x:c>
+      <x:c r="C20" s="18" t="str">
+        <x:v>原始切片／成本輸入。CTB 檔案內容不變。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="28" customHeight="1">
+      <x:c r="A21" s="18" t="str">
+        <x:v>原始公式</x:v>
+      </x:c>
+      <x:c r="B21" s="18" t="str">
+        <x:v>NTD = 1.2 × (25 + original resin subtotal × 1.1 + estimated printing hours × 7.195).</x:v>
+      </x:c>
+      <x:c r="C21" s="18" t="str">
+        <x:v>NTD 原始公式。成本已包含原公式的機器項，不另加一瓶樹脂或機器重購成本。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="96" customHeight="1">
+      <x:c r="A22" s="18" t="str">
+        <x:v>P1: 01</x:v>
+      </x:c>
+      <x:c r="B22" s="18" t="str">
+        <x:v>Material: PC/GF-like Black
+Time: 17 h 35 min (1055 min)
+Resin volume: 107.531 mL; mass: 118.285 g
+Original resin quotation: NTD 260.226
+Original reported total: NTD 525.313
+Recomputed source-formula total: NTD 525.31282</x:v>
+      </x:c>
+      <x:c r="C22" s="18" t="str">
+        <x:v>原始報價備查；採用 Print_batches 的完整精度公式結果。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="96" customHeight="1">
+      <x:c r="A23" s="18" t="str">
+        <x:v>P2: 02 + 03 + 08</x:v>
+      </x:c>
+      <x:c r="B23" s="18" t="str">
+        <x:v>Material: PC/GF-like Black
+Time: 16 h 19 min (979 min)
+Resin volume: 114.027 mL; mass: 125.43 g
+Original resin quotation: NTD 275.945
+Original reported total: NTD 535.126
+Recomputed source-formula total: NTD 535.1255</x:v>
+      </x:c>
+      <x:c r="C23" s="18" t="str">
+        <x:v>原始報價備查；採用 Print_batches 的完整精度公式結果。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="96" customHeight="1">
+      <x:c r="A24" s="18" t="str">
+        <x:v>P3: 04 + 05 + 06 + 07</x:v>
+      </x:c>
+      <x:c r="B24" s="18" t="str">
+        <x:v>Material: Aqua Clear Plus
+Time: 2 h 42 min (162 min)
+Resin volume: 1.198 mL; mass: 1.318 g
+Original resin quotation: NTD 1.239
+Original reported total: NTD 52.215
+Recomputed source-formula total: NTD 54.94728</x:v>
+      </x:c>
+      <x:c r="C24" s="18" t="str">
+        <x:v>原始報價備查；採用 Print_batches 的完整精度公式結果。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="40" customHeight="1">
+      <x:c r="A25" s="18" t="str">
+        <x:v>P3 原報差異</x:v>
+      </x:c>
+      <x:c r="B25" s="18" t="str">
+        <x:v>透明井批次原報 NTD 52.215；原輸入與公式算得 NTD 54.94728。預算使用公式結果。P1/P2 的原報差異屬四捨五入。</x:v>
+      </x:c>
+      <x:c r="C25" s="18" t="str"/>
+    </x:row>
+    <x:row r="26" ht="40" customHeight="1">
+      <x:c r="A26" s="18" t="str">
+        <x:v>精度與來源識別</x:v>
+      </x:c>
+      <x:c r="B26" s="18" t="str">
+        <x:v>三批完整精度相加後才顯示兩位小數。合印批次不假造個別零件價格。</x:v>
+      </x:c>
+      <x:c r="C26" s="18" t="str">
+        <x:v>Original print-cost record SHA256: 174599bf359f0186bfe581aab6033953525edf30911b7083e27cb033251b24dd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="30" customHeight="1">
+      <x:c r="A27" s="25" t="str">
+        <x:v>價格來源總表</x:v>
+      </x:c>
+      <x:c r="B27" s="25" t="str"/>
+      <x:c r="C27" s="25" t="str"/>
+    </x:row>
+    <x:row r="28" ht="54" customHeight="1">
+      <x:c r="A28" s="18" t="str">
+        <x:v>FX</x:v>
+      </x:c>
+      <x:c r="B28" s="18" t="str">
+        <x:v>Bank of Taiwan USD spot selling
+2026-10-05 15:13 displayed snapshot: USD spot buy 31.705, sell 31.805. Budget conversion uses sell 31.805, not an October 8 live execution quote.</x:v>
+      </x:c>
+      <x:c r="C28" s="18" t="str">
+        <x:v>https://www.bot.com.tw/tw/personal-banking/foreign-exchange</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="40" customHeight="1">
+      <x:c r="A29" s="18" t="str">
+        <x:v>FAN</x:v>
+      </x:c>
+      <x:c r="B29" s="18" t="str">
+        <x:v>DigiKey MF40100V1-1000U-A99
+NTD 161 at quantity 1. Listed out of stock. Shipping and local tax not added.</x:v>
+      </x:c>
+      <x:c r="C29" s="18" t="str">
+        <x:v>https://www.digikey.tw/en/products/detail/sunon-fans/MF40100V1-1000U-A99/6198732</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="68" customHeight="1">
+      <x:c r="A30" s="18" t="str">
+        <x:v>FASTENER</x:v>
+      </x:c>
+      <x:c r="B30" s="18" t="str">
+        <x:v>Local small-fastener retail benchmark
+Listing shows small M3 fasteners around NTD 3 individually. Listed flat-head type is NOT the specified socket cap. Budget allowances 3/4/6 NTD for M3x8/16/35 cap screws, 2 for nuts and 1 for washers; local exact-type prices unverified.</x:v>
+      </x:c>
+      <x:c r="C30" s="18" t="str">
+        <x:v>https://www.ruten.com.tw/item/21306183365097/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="54" customHeight="1">
+      <x:c r="A31" s="18" t="str">
+        <x:v>SEAL</x:v>
+      </x:c>
+      <x:c r="B31" s="18" t="str">
+        <x:v>Black silicone sheet size reference
+0.8 mm selectable stock; exact price unavailable. NTD 150 per small sheet is an engineering allowance, not a verified selling price. Hardness and VOC compatibility unqualified.</x:v>
+      </x:c>
+      <x:c r="C31" s="18" t="str">
+        <x:v>https://www.ruten.com.tw/item/22517308416481/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="54" customHeight="1">
+      <x:c r="A32" s="18" t="str">
+        <x:v>POWER</x:v>
+      </x:c>
+      <x:c r="B32" s="18" t="str">
+        <x:v>Adafruit 4298 USB-C supply
+USD 8.74, 5.1 V 3 A with cable. Price benchmark only; vendor must confirm input and charging configuration. Current budget uses external power, not an unconfirmed battery.</x:v>
+      </x:c>
+      <x:c r="C32" s="18" t="str">
+        <x:v>https://www.adafruit.com/product/4298</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="68" customHeight="1">
+      <x:c r="A33" s="18" t="str">
+        <x:v>GASFILTER</x:v>
+      </x:c>
+      <x:c r="B33" s="18" t="str">
+        <x:v>Gilson ANP1322 SupaTop
+USD 95 per 100. Hydrophobic PTFE, 13 mm, 0.22 um, NONSTERILE, air venting listed. Price proxy for 0.2 um gas-filter requirement, not certified sterile replacement. Two used per device; buying a box costs 100 filters.</x:v>
+      </x:c>
+      <x:c r="C33" s="18" t="str">
+        <x:v>https://www.gilson.com/default/catalog/product/view/id/1204/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="54" customHeight="1">
+      <x:c r="A34" s="18" t="str">
+        <x:v>PTFE</x:v>
+      </x:c>
+      <x:c r="B34" s="18" t="str">
+        <x:v>Tinkersphere 2 mm ID 3 mm OD PTFE
+Search listing USD 4.99; sold length not verified. NTD 200 per 1 m is a separate allowance. Printer-feed tubing is not qualified analytical tubing.</x:v>
+      </x:c>
+      <x:c r="C34" s="18" t="str">
+        <x:v>https://tinkersphere.com/3d-printer-parts-supplies/2015-ptfe-teflon-tube-2mm-id-3mm-od-for-175-mm-filament.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="54" customHeight="1">
+      <x:c r="A35" s="18" t="str">
+        <x:v>COUPLER</x:v>
+      </x:c>
+      <x:c r="B35" s="18" t="str">
+        <x:v>Adafruit 3 mm ID silicone tubing reference
+Related tubing listed USD 2.50 per metre. Budget NTD 150 includes short flexible couplers and matching adapters. Exact ID/OD, Luer interfaces and VOC recovery must be checked; no fit guarantee.</x:v>
+      </x:c>
+      <x:c r="C35" s="18" t="str">
+        <x:v>https://www.adafruit.com/product/4699</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="68" customHeight="1">
+      <x:c r="A36" s="18" t="str">
+        <x:v>OPTIC</x:v>
+      </x:c>
+      <x:c r="B36" s="18" t="str">
+        <x:v>Edmund Optics 67-016 520 nm emission filter
+USD 284, 12.5 mm diameter, substrate 2.00 +/-0.25 mm, mounted. Does NOT fit 5.2x4.2x1.0 mm seat. NTD 12000 is a custom thin-filter budget allowance, not a quote or available drop-in part. Cutting this stock part does not solve its thickness mismatch.</x:v>
+      </x:c>
+      <x:c r="C36" s="18" t="str">
+        <x:v>https://www.edmundoptics.com/p/520nm-cwl-125mm-dia-36nm-bandwidth-od-6-fluorescence-filter/21556/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="54" customHeight="1">
+      <x:c r="A37" s="18" t="str">
+        <x:v>UART</x:v>
+      </x:c>
+      <x:c r="B37" s="18" t="str">
+        <x:v>Adafruit 5335 CP2102N Friend
+USD 5.95 each. Signals 3.3 V; power wire 5 V. Leave VCC disconnected at J3. Cable and jumper wires separate.</x:v>
+      </x:c>
+      <x:c r="C37" s="18" t="str">
+        <x:v>https://www.adafruit.com/product/5335</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="68" customHeight="1">
+      <x:c r="A38" s="18" t="str">
+        <x:v>PUMP</x:v>
+      </x:c>
+      <x:c r="B38" s="18" t="str">
+        <x:v>Adafruit 4699 gas pump price benchmark
+USD 7.95 for pump alone. 2.5 L/min, intermittent duty; NOT a selected 3 mL/min continuous source. NTD 5000 system allowance requires a qualified controlled source, bypass/regulation, pressure protection, fittings and supply. Borrow a suitable lab system first.</x:v>
+      </x:c>
+      <x:c r="C38" s="18" t="str">
+        <x:v>https://www.adafruit.com/product/4699</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="68" customHeight="1">
+      <x:c r="A39" s="18" t="str">
+        <x:v>FLOW</x:v>
+      </x:c>
+      <x:c r="B39" s="18" t="str">
+        <x:v>Omega precision rotameter range reference
+FL-320 nominal air range 0.02-15 cc/min. Historical price deliberately not treated as current. NTD 15000 is a planning allowance pending current calibrated meter quote; 3 mL/min must fall within usable range.</x:v>
+      </x:c>
+      <x:c r="C39" s="18" t="str">
+        <x:v>https://br.omega.com/omegaFiles/green/pdf/FL120.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="54" customHeight="1">
+      <x:c r="A40" s="18" t="str">
+        <x:v>DYE</x:v>
+      </x:c>
+      <x:c r="B40" s="18" t="str">
+        <x:v>Sigma 46970 sodium fluorescein
+USD 52.60 per 100 g. Budget includes whole bottle, not a fictitious single-well quantity. Prefer a documented laboratory aliquot. Not an assay-specific or GCaMP-certified standard.</x:v>
+      </x:c>
+      <x:c r="C40" s="18" t="str">
+        <x:v>https://www.sigmaaldrich.com/US/en/product/sigma/46970</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="54" customHeight="1">
+      <x:c r="A41" s="18" t="str">
+        <x:v>VALVE</x:v>
+      </x:c>
+      <x:c r="B41" s="18" t="str">
+        <x:v>Adafruit 4663 FA0520E
+USD 2.95 for 6 V valve alone. NTD 500 system allowance includes driver, flyback diode, supply and fittings. Future only; VOC wetted-material suitability and firmware support unverified.</x:v>
+      </x:c>
+      <x:c r="C41" s="18" t="str">
+        <x:v>https://www.adafruit.com/product/4663</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="54" customHeight="1">
+      <x:c r="A42" s="18" t="str">
+        <x:v>PDMS</x:v>
+      </x:c>
+      <x:c r="B42" s="18" t="str">
+        <x:v>Dow Sylgard 184 0.5 kg kit reference
+Kit identity found; current public price not verified. NTD 6000 planning allowance for kit and basic casting consumables. No claim that PDMS removes water selectively.</x:v>
+      </x:c>
+      <x:c r="C42" s="18" t="str">
+        <x:v>https://labproinc.com/products/dow-sylgard-184-silicone-encapsulant-clear-0-5-kg-kit-184-sil-elast-kit-0-5kg</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="68" customHeight="1">
+      <x:c r="A43" s="18" t="str">
+        <x:v>TOOLS</x:v>
+      </x:c>
+      <x:c r="B43" s="18" t="str">
+        <x:v>Local tools and lab access allowance
+Engineering allowances only: hand tools/calipers NTD 1500; DMM 800; scope 10000; pipette/tips 4000; print/post-cure supplies 300. Borrow existing printer, wash/cure equipment, PC, phone, biosafety/cell facilities. Their capital replacement prices are outside this BOM.</x:v>
+      </x:c>
+      <x:c r="C43" s="18" t="str">
+        <x:v>Original planning record; no public price URL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="40" customHeight="1">
+      <x:c r="A44" s="18" t="str">
+        <x:v>PCB_LED</x:v>
+      </x:c>
+      <x:c r="B44" s="18" t="str">
+        <x:v>DigiKey 155124BS73200
+NTD 17 each at quantity 1.</x:v>
+      </x:c>
+      <x:c r="C44" s="18" t="str">
+        <x:v>https://www.digikey.tw/en/products/detail/w%C3%BCrth-elektronik/155124BS73200/4490035</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="40" customHeight="1">
+      <x:c r="A45" s="18" t="str">
+        <x:v>PCB_PD</x:v>
+      </x:c>
+      <x:c r="B45" s="18" t="str">
+        <x:v>DigiKey VEMD5060X01
+NTD 68 each at quantity 1.</x:v>
+      </x:c>
+      <x:c r="C45" s="18" t="str">
+        <x:v>https://www.digikey.tw/en/products/detail/vishay-semiconductor-opto-division/VEMD5060X01/5879084</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="54" customHeight="1">
+      <x:c r="A46" s="18" t="str">
+        <x:v>PCB_U1</x:v>
+      </x:c>
+      <x:c r="B46" s="18" t="str">
+        <x:v>DigiKey TPS61023 family
+Search results list TPS61023DRLT cut tape NTD 52. Packaging-suffix proxy for vendor TPS61023; exact order code requires confirmation.</x:v>
+      </x:c>
+      <x:c r="C46" s="18" t="str">
+        <x:v>https://www.digikey.tw/en/products/detail/texas-instruments/TPS61023DRLR/11310629</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="40" customHeight="1">
+      <x:c r="A47" s="18" t="str">
+        <x:v>PCB_U2</x:v>
+      </x:c>
+      <x:c r="B47" s="18" t="str">
+        <x:v>DigiKey BQ24074RGTR
+NTD 88 each at quantity 1; RGT package assumed from schematic.</x:v>
+      </x:c>
+      <x:c r="C47" s="18" t="str">
+        <x:v>https://www.digikey.tw/en/products/detail/texas-instruments/BQ24074RGTR/2047269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="40" customHeight="1">
+      <x:c r="A48" s="18" t="str">
+        <x:v>PCB_U4</x:v>
+      </x:c>
+      <x:c r="B48" s="18" t="str">
+        <x:v>DigiKey ESP32-WROOM-32E-N4
+NTD 181 each. N4 is a price proxy; vendor flash suffix missing.</x:v>
+      </x:c>
+      <x:c r="C48" s="18" t="str">
+        <x:v>https://www.digikey.tw/en/products/detail/espressif-systems/ESP32-WROOM-32E-N4/11613125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="40" customHeight="1">
+      <x:c r="A49" s="18" t="str">
+        <x:v>PCB_U6</x:v>
+      </x:c>
+      <x:c r="B49" s="18" t="str">
+        <x:v>DigiKey LP5907MFX-3.3/NOPB
+NTD 24 each at quantity 1.</x:v>
+      </x:c>
+      <x:c r="C49" s="18" t="str">
+        <x:v>https://www.digikey.tw/en/products/detail/texas-instruments/LP5907MFX-3-3-NOPB/3906441</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="40" customHeight="1">
+      <x:c r="A50" s="18" t="str">
+        <x:v>PCB_U7</x:v>
+      </x:c>
+      <x:c r="B50" s="18" t="str">
+        <x:v>DigiKey LTC6655BHMS8-2.5#TRPBF
+NTD 628 for cut tape. Packaging proxy for #PBF; listed no stock.</x:v>
+      </x:c>
+      <x:c r="C50" s="18" t="str">
+        <x:v>https://www.digikey.tw/en/products/detail/analog-devices-inc/LTC6655BHMS8-2-5-TRPBF/2181717</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="40" customHeight="1">
+      <x:c r="A51" s="18" t="str">
+        <x:v>PCB_U8</x:v>
+      </x:c>
+      <x:c r="B51" s="18" t="str">
+        <x:v>DigiKey LMP7721MAX/NOPB listing
+Search listing NTD 226 for MAX/NOPB. Vendor LMP7721 suffix missing; package proxy.</x:v>
+      </x:c>
+      <x:c r="C51" s="18" t="str">
+        <x:v>https://www.digikey.tw/en/products/filter/linear/amplifiers/instrumentation-op-amps-buffer-amps/687</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="40" customHeight="1">
+      <x:c r="A52" s="18" t="str">
+        <x:v>PCB_U9</x:v>
+      </x:c>
+      <x:c r="B52" s="18" t="str">
+        <x:v>DigiKey ADS8866IDGS
+NTD 306 each at quantity 1.</x:v>
+      </x:c>
+      <x:c r="C52" s="18" t="str">
+        <x:v>https://www.digikey.tw/zh/products/detail/texas-instruments/ADS8866IDGS/5176196</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="82" customHeight="1">
+      <x:c r="A53" s="18" t="str">
+        <x:v>PCB_MISC</x:v>
+      </x:c>
+      <x:c r="B53" s="18" t="str">
+        <x:v>Unspecified PCB parts allowance
+Generic single-piece budgets, NOT verified quotations: small resistors NTD 1, high-value resistor 30, shunt 5; ceramics 2-8; bulk capacitor 15; LED 2; MOSFET 5; inductor 10; connectors 5-30; switches 5-15; linear regulator 10. Unknown U3 remains unpriced. Do not purchase substitutes without vendor values, packages and ratings.</x:v>
+      </x:c>
+      <x:c r="C53" s="18" t="str">
+        <x:v>Original planning record; no public price URL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="30" customHeight="1">
+      <x:c r="A54" s="25" t="str">
+        <x:v>規格來源總表</x:v>
+      </x:c>
+      <x:c r="B54" s="25" t="str"/>
+      <x:c r="C54" s="25" t="str"/>
+    </x:row>
+    <x:row r="55" ht="28" customHeight="1">
+      <x:c r="A55" s="18" t="str">
+        <x:v>procurement: CAD</x:v>
+      </x:c>
+      <x:c r="B55" s="18" t="str">
+        <x:v>Existing frozen geometry; read-only audit, no changes.</x:v>
+      </x:c>
+      <x:c r="C55" s="18" t="str">
+        <x:v>原始來源識別：09_engineering_sources/CAD/aerosense.scad</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="28" customHeight="1">
+      <x:c r="A56" s="18" t="str">
+        <x:v>procurement: STL</x:v>
+      </x:c>
+      <x:c r="B56" s="18" t="str">
+        <x:v>All8 binary STL bounds independently read; exported Z minima are0. Assembly coordinates are separate.</x:v>
+      </x:c>
+      <x:c r="C56" s="18" t="str">
+        <x:v>原始來源識別：01_print</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="28" customHeight="1">
+      <x:c r="A57" s="18" t="str">
+        <x:v>procurement: ASM</x:v>
+      </x:c>
+      <x:c r="B57" s="18" t="str"/>
+      <x:c r="C57" s="18" t="str">
+        <x:v>原始來源識別：04_manuals/Assembly_Manual_ZH.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="28" customHeight="1">
+      <x:c r="A58" s="18" t="str">
+        <x:v>procurement: GASKET</x:v>
+      </x:c>
+      <x:c r="B58" s="18" t="str"/>
+      <x:c r="C58" s="18" t="str">
+        <x:v>原始來源識別：09_engineering_sources/CAD/drawings/gasket_cut_template_1to1.svg</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="28" customHeight="1">
+      <x:c r="A59" s="18" t="str">
+        <x:v>procurement: FLOW</x:v>
+      </x:c>
+      <x:c r="B59" s="18" t="str"/>
+      <x:c r="C59" s="18" t="str">
+        <x:v>原始來源識別：02_simulation/airflow/Flow_Operation_ZH.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="28" customHeight="1">
+      <x:c r="A60" s="18" t="str">
+        <x:v>procurement: OPTICS</x:v>
+      </x:c>
+      <x:c r="B60" s="18" t="str"/>
+      <x:c r="C60" s="18" t="str">
+        <x:v>原始來源識別：02_simulation/optics/Analysis_EN.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="28" customHeight="1">
+      <x:c r="A61" s="18" t="str">
+        <x:v>procurement: OPERATION</x:v>
+      </x:c>
+      <x:c r="B61" s="18" t="str"/>
+      <x:c r="C61" s="18" t="str">
+        <x:v>原始來源識別：03_software/guides/Operation_and_Setup_EN.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="28" customHeight="1">
+      <x:c r="A62" s="18" t="str">
+        <x:v>procurement: VALIDATION</x:v>
+      </x:c>
+      <x:c r="B62" s="18" t="str"/>
+      <x:c r="C62" s="18" t="str">
+        <x:v>原始來源識別：07_validation/Fluorescence_and_Cell_Test_ZH.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="28" customHeight="1">
+      <x:c r="A63" s="18" t="str">
+        <x:v>procurement: ELEC</x:v>
+      </x:c>
+      <x:c r="B63" s="18" t="str">
+        <x:v>Schematic interpretation supplied by optics audit agent2026-10-06; value/MPN uncertainties retained.</x:v>
+      </x:c>
+      <x:c r="C63" s="18" t="str">
+        <x:v>原始來源識別：08_reference/NTHU_TEST_BOARD_Schematic.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="28" customHeight="1">
+      <x:c r="A64" s="18" t="str">
+        <x:v>procurement: FAN</x:v>
+      </x:c>
+      <x:c r="B64" s="18" t="str">
+        <x:v>Official SUNON catalogue,printed p32/PDF p32; candidate5V136mA0.68W;frame40±0.5,pitch32±0.3.</x:v>
+      </x:c>
+      <x:c r="C64" s="18" t="str">
+        <x:v>https://www.sunon.com/eu/MANAGE/Docs/WEBCONT/Files/1236/DC%20Fan_20240630(255-E)_s.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="40" customHeight="1">
+      <x:c r="A65" s="18" t="str">
+        <x:v>procurement: SCREW</x:v>
+      </x:c>
+      <x:c r="B65" s="18" t="str">
+        <x:v>Official Bossard M3 ISO4762/DIN912 dimensional reference:head5.5,height3,hex2.5. This30-mm article is a family-dimension reference,not a purchased length or MPN selection.</x:v>
+      </x:c>
+      <x:c r="C65" s="18" t="str">
+        <x:v>https://nederland.bossard.com/en-us/standard-fastening-elements/screws/screws-and-bolts-with-internal-drive/912000a20030030</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="28" customHeight="1">
+      <x:c r="A66" s="18" t="str">
+        <x:v>procurement: PITCH</x:v>
+      </x:c>
+      <x:c r="B66" s="18" t="str">
+        <x:v>Official KIPP coarse metric pitch:M3×0.5.</x:v>
+      </x:c>
+      <x:c r="C66" s="18" t="str">
+        <x:v>https://www.kippusa.com/en-us/measurement-units</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="40" customHeight="1">
+      <x:c r="A67" s="18" t="str">
+        <x:v>procurement: NUT</x:v>
+      </x:c>
+      <x:c r="B67" s="18" t="str">
+        <x:v>Bossard manufacturer datasheet hosted by distributor,BN629 DIN934/~ISO4032:M3,AF5.5,height max2.4. Dimensional evidence,not selected MPN.</x:v>
+      </x:c>
+      <x:c r="C67" s="18" t="str">
+        <x:v>https://media.distrelec.com/Web/Downloads/_t/ds/1241613_eng_tds.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="40" customHeight="1">
+      <x:c r="A68" s="18" t="str">
+        <x:v>procurement: WASHER</x:v>
+      </x:c>
+      <x:c r="B68" s="18" t="str">
+        <x:v>Direct supplier dimensional reference:ID3.2/OD7/thickness0.5. Nylon article is not a final material/MPN selection; PCB insulation choice remains open.</x:v>
+      </x:c>
+      <x:c r="C68" s="18" t="str">
+        <x:v>https://www.accu.co.uk/metric-flat-washers/465682-HPW-3-2-7-0-5-N</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="54" customHeight="1">
+      <x:c r="A69" s="18" t="str">
+        <x:v>PCB: vendor_BOM</x:v>
+      </x:c>
+      <x:c r="B69" s="18" t="str">
+        <x:v>NTHU_TEST_BOARD_BOM.docx, vendor table, 61 rows
+Accessed: 2026-10-06
+SHA256: 3541da4a10afbfc371f4ec7c8094329fea7ed84635b543628252fe67276fa4b8</x:v>
+      </x:c>
+      <x:c r="C69" s="18" t="str">
+        <x:v>原始來源識別：08_reference/NTHU_TEST_BOARD_BOM.docx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="54" customHeight="1">
+      <x:c r="A70" s="18" t="str">
+        <x:v>PCB: schematic</x:v>
+      </x:c>
+      <x:c r="B70" s="18" t="str">
+        <x:v>NTHU_TEST_BOARD_Schematic.pdf, version A, 14 September 2026, sheets 1–2
+Accessed: 2026-10-06
+SHA256: c8cfc0600a6d34740c1caac24f37d9eaea6bea59b88278e4258988769939d07e</x:v>
+      </x:c>
+      <x:c r="C70" s="18" t="str">
+        <x:v>原始來源識別：08_reference/NTHU_TEST_BOARD_Schematic.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="40" customHeight="1">
+      <x:c r="A71" s="18" t="str">
+        <x:v>PCB: TI_TPS61023</x:v>
+      </x:c>
+      <x:c r="B71" s="18" t="str">
+        <x:v>Texas Instruments TPS61023 product information
+Accessed: 2026-10-06</x:v>
+      </x:c>
+      <x:c r="C71" s="18" t="str">
+        <x:v>https://www.ti.com/product/TPS61023</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="40" customHeight="1">
+      <x:c r="A72" s="18" t="str">
+        <x:v>PCB: TI_BQ24074</x:v>
+      </x:c>
+      <x:c r="B72" s="18" t="str">
+        <x:v>Texas Instruments BQ24074 product information
+Accessed: 2026-10-06</x:v>
+      </x:c>
+      <x:c r="C72" s="18" t="str">
+        <x:v>https://www.ti.com/product/BQ24074</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="40" customHeight="1">
+      <x:c r="A73" s="18" t="str">
+        <x:v>PCB: TI_LP5907</x:v>
+      </x:c>
+      <x:c r="B73" s="18" t="str">
+        <x:v>Texas Instruments LP5907 datasheet, ordering/package information
+Accessed: 2026-10-06</x:v>
+      </x:c>
+      <x:c r="C73" s="18" t="str">
+        <x:v>https://www.ti.com/lit/ds/symlink/lp5907.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="40" customHeight="1">
+      <x:c r="A74" s="18" t="str">
+        <x:v>PCB: TI_LMP7721</x:v>
+      </x:c>
+      <x:c r="B74" s="18" t="str">
+        <x:v>Texas Instruments LMP7721 product information
+Accessed: 2026-10-06</x:v>
+      </x:c>
+      <x:c r="C74" s="18" t="str">
+        <x:v>https://www.ti.com/product/LMP7721</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="40" customHeight="1">
+      <x:c r="A75" s="18" t="str">
+        <x:v>PCB: TI_ADS8866</x:v>
+      </x:c>
+      <x:c r="B75" s="18" t="str">
+        <x:v>Texas Instruments ADS8866 datasheet, ADS8866IDGS ordering information
+Accessed: 2026-10-06</x:v>
+      </x:c>
+      <x:c r="C75" s="18" t="str">
+        <x:v>https://www.ti.com/lit/ds/symlink/ads8866.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="40" customHeight="1">
+      <x:c r="A76" s="18" t="str">
+        <x:v>PCB: ADI_LTC6655</x:v>
+      </x:c>
+      <x:c r="B76" s="18" t="str">
+        <x:v>Analog Devices LTC6655 / LTC6655LN datasheet
+Accessed: 2026-10-06</x:v>
+      </x:c>
+      <x:c r="C76" s="18" t="str">
+        <x:v>https://www.analog.com/media/en/technical-documentation/data-sheets/LTC6655-6655LN.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="40" customHeight="1">
+      <x:c r="A77" s="18" t="str">
+        <x:v>PCB: ECMOS_EC50117</x:v>
+      </x:c>
+      <x:c r="B77" s="18" t="str">
+        <x:v>E-CMOS EC50117 datasheet 9L05N Rev F004; page 2 EC50117KBG ordering row
+Accessed: 2026-10-06</x:v>
+      </x:c>
+      <x:c r="C77" s="18" t="str">
+        <x:v>https://www.ecmos.com.tw/wp-content/uploads/2022/07/EC50117_9L05N-Rev.F004.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="40" customHeight="1">
+      <x:c r="A78" s="18" t="str">
+        <x:v>PCB: ESPRESSIF_32E</x:v>
+      </x:c>
+      <x:c r="B78" s="18" t="str">
+        <x:v>Espressif ESP32-WROOM-32E / ESP32-WROOM-32UE datasheet
+Accessed: 2026-10-06</x:v>
+      </x:c>
+      <x:c r="C78" s="18" t="str">
+        <x:v>https://www.espressif.com/sites/default/files/documentation/esp32-wroom-32e_esp32-wroom-32ue_datasheet_en.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="40" customHeight="1">
+      <x:c r="A79" s="18" t="str">
+        <x:v>PCB: WURTH_LED</x:v>
+      </x:c>
+      <x:c r="B79" s="18" t="str">
+        <x:v>Würth Elektronik 155124BS73200 datasheet
+Accessed: 2026-10-06</x:v>
+      </x:c>
+      <x:c r="C79" s="18" t="str">
+        <x:v>https://www.we-online.com/components/products/datasheet/155124BS73200.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="40" customHeight="1">
+      <x:c r="A80" s="18" t="str">
+        <x:v>PCB: VISHAY_PD</x:v>
+      </x:c>
+      <x:c r="B80" s="18" t="str">
+        <x:v>Vishay VEMD5060X01 product information, document 84278
+Accessed: 2026-10-06</x:v>
+      </x:c>
+      <x:c r="C80" s="18" t="str">
+        <x:v>https://www.vishay.com/en/product/84278/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="40" customHeight="1">
+      <x:c r="A81" s="18" t="str">
+        <x:v>PCB: AOS_AO3400A</x:v>
+      </x:c>
+      <x:c r="B81" s="18" t="str">
+        <x:v>Alpha &amp; Omega Semiconductor AO3400A datasheet
+Accessed: 2026-10-06</x:v>
+      </x:c>
+      <x:c r="C81" s="18" t="str">
+        <x:v>https://www.aosmd.com/res/data_sheets/AO3400A.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="30" customHeight="1">
+      <x:c r="A82" s="25" t="str">
+        <x:v>採購補充來源</x:v>
+      </x:c>
+      <x:c r="B82" s="25" t="str"/>
+      <x:c r="C82" s="25" t="str"/>
+    </x:row>
+    <x:row r="83" ht="28" customHeight="1">
+      <x:c r="A83" s="18" t="str">
+        <x:v>歷史欄位</x:v>
+      </x:c>
+      <x:c r="B83" s="18" t="str">
+        <x:v>以下保留料號、原始来源欄位與早期估值，不取代目前價格輸入，也不另外加總。</x:v>
+      </x:c>
+      <x:c r="C83" s="18" t="str"/>
+    </x:row>
+    <x:row r="84" ht="96" customHeight="1">
+      <x:c r="A84" s="18" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B84" s="18" t="str">
+        <x:v>price_source: FAN
+source: RS 2025400 viewed 2026-09-24 incl tax; out of stock then. https://twcn.rs-online.com/web/p/axial-fans/2025400
+low: 161
+high: 161
+source_zh: CAD; ASM; FAN</x:v>
+      </x:c>
+      <x:c r="C84" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="82" customHeight="1">
+      <x:c r="A85" s="18" t="str">
+        <x:v>H01</x:v>
+      </x:c>
+      <x:c r="B85" s="18" t="str">
+        <x:v>price_source: FASTENER
+source: Quotation pending; no invented price / 尚待報價，未填假價格
+low: 3
+high: 3
+source_zh: CAD; ASM; SCREW; PITCH</x:v>
+      </x:c>
+      <x:c r="C85" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="82" customHeight="1">
+      <x:c r="A86" s="18" t="str">
+        <x:v>H02</x:v>
+      </x:c>
+      <x:c r="B86" s="18" t="str">
+        <x:v>price_source: FASTENER
+source: Quotation pending; no invented price / 尚待報價，未填假價格
+low: 4
+high: 4
+source_zh: CAD; ASM; SCREW; PITCH</x:v>
+      </x:c>
+      <x:c r="C86" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="82" customHeight="1">
+      <x:c r="A87" s="18" t="str">
+        <x:v>H03</x:v>
+      </x:c>
+      <x:c r="B87" s="18" t="str">
+        <x:v>price_source: FASTENER
+source: Quotation pending; no invented price / 尚待報價，未填假價格
+low: 6
+high: 6
+source_zh: CAD; ASM; SCREW; PITCH</x:v>
+      </x:c>
+      <x:c r="C87" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="82" customHeight="1">
+      <x:c r="A88" s="18" t="str">
+        <x:v>H04</x:v>
+      </x:c>
+      <x:c r="B88" s="18" t="str">
+        <x:v>price_source: FASTENER
+source: Planning allowance, NOT supplier quote / 預算假設，非報價
+low: 2
+high: 2
+source_zh: CAD; ASM; NUT</x:v>
+      </x:c>
+      <x:c r="C88" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="82" customHeight="1">
+      <x:c r="A89" s="18" t="str">
+        <x:v>H05</x:v>
+      </x:c>
+      <x:c r="B89" s="18" t="str">
+        <x:v>price_source: FASTENER
+source: Planning allowance, NOT supplier quote / 預算假設，非報價
+low: 1
+high: 1
+source_zh: CAD; ASM; WASHER</x:v>
+      </x:c>
+      <x:c r="C89" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="82" customHeight="1">
+      <x:c r="A90" s="18" t="str">
+        <x:v>E01</x:v>
+      </x:c>
+      <x:c r="B90" s="18" t="str">
+        <x:v>price_source: TOOLS
+source: Planning allowance, NOT supplier quote / 預算假設，非報價
+low: 80
+high: 80
+source_zh: ASM; ELEC</x:v>
+      </x:c>
+      <x:c r="C90" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="82" customHeight="1">
+      <x:c r="A91" s="18" t="str">
+        <x:v>S01</x:v>
+      </x:c>
+      <x:c r="B91" s="18" t="str">
+        <x:v>price_source: SEAL
+source: Planning allowance, NOT supplier quote / 預算假設，非報價
+low: 150
+high: 150
+source_zh: CAD; ASM; GASKET</x:v>
+      </x:c>
+      <x:c r="C91" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="82" customHeight="1">
+      <x:c r="A92" s="18" t="str">
+        <x:v>E02</x:v>
+      </x:c>
+      <x:c r="B92" s="18" t="str">
+        <x:v>price_source: POWER
+source: Quotation pending; no invented price / 尚待報價，未填假價格
+low: 277.9757
+high: 277.9757
+source_zh: ELEC; ASM</x:v>
+      </x:c>
+      <x:c r="C92" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="82" customHeight="1">
+      <x:c r="A93" s="18" t="str">
+        <x:v>G01</x:v>
+      </x:c>
+      <x:c r="B93" s="18" t="str">
+        <x:v>price_source: GASFILTER
+source: Quotation pending; no invented price / 尚待報價，未填假價格
+low: 30.21475
+high: 30.21475
+source_zh: ASM; FLOW</x:v>
+      </x:c>
+      <x:c r="C93" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="82" customHeight="1">
+      <x:c r="A94" s="18" t="str">
+        <x:v>G02</x:v>
+      </x:c>
+      <x:c r="B94" s="18" t="str">
+        <x:v>price_source: PTFE
+source: Planning allowance, NOT supplier quote / 預算假設，非報價
+low: 200
+high: 200
+source_zh: CAD; ASM; FLOW</x:v>
+      </x:c>
+      <x:c r="C94" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="82" customHeight="1">
+      <x:c r="A95" s="18" t="str">
+        <x:v>G03</x:v>
+      </x:c>
+      <x:c r="B95" s="18" t="str">
+        <x:v>price_source: COUPLER
+source: Quotation pending; no invented price / 尚待報價，未填假價格
+low: 150
+high: 150
+source_zh: CAD; ASM</x:v>
+      </x:c>
+      <x:c r="C95" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="82" customHeight="1">
+      <x:c r="A96" s="18" t="str">
+        <x:v>O01</x:v>
+      </x:c>
+      <x:c r="B96" s="18" t="str">
+        <x:v>price_source: OPTIC
+source: Quotation pending; no invented price / 尚待報價，未填假價格
+low: 12000
+high: 12000
+source_zh: CAD; ASM; OPTICS</x:v>
+      </x:c>
+      <x:c r="C96" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="82" customHeight="1">
+      <x:c r="A97" s="18" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="B97" s="18" t="str">
+        <x:v>price_source: UART
+source: Quotation pending; no invented price / 尚待報價，未填假價格
+low: 189.23975000000002
+high: 189.23975000000002
+source_zh: OPERATION; ELEC</x:v>
+      </x:c>
+      <x:c r="C97" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="82" customHeight="1">
+      <x:c r="A98" s="18" t="str">
+        <x:v>L01</x:v>
+      </x:c>
+      <x:c r="B98" s="18" t="str">
+        <x:v>price_source: PUMP
+source: Quotation pending; no invented price / 尚待報價，未填假價格
+low: 5000
+high: 5000
+source_zh: ASM; FLOW</x:v>
+      </x:c>
+      <x:c r="C98" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="82" customHeight="1">
+      <x:c r="A99" s="18" t="str">
+        <x:v>L02</x:v>
+      </x:c>
+      <x:c r="B99" s="18" t="str">
+        <x:v>price_source: TOOLS
+source: Quotation pending; no invented price / 尚待報價，未填假價格
+low: 1500
+high: 1500
+source_zh: ASM; SCREW</x:v>
+      </x:c>
+      <x:c r="C99" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="82" customHeight="1">
+      <x:c r="A100" s="18" t="str">
+        <x:v>L03</x:v>
+      </x:c>
+      <x:c r="B100" s="18" t="str">
+        <x:v>price_source: DYE
+source: Quotation pending; no invented price / 尚待報價，未填假價格
+low: 1672.943
+high: 1672.943
+source_zh: VALIDATION; OPERATION</x:v>
+      </x:c>
+      <x:c r="C100" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="40" customHeight="1">
+      <x:c r="A101" s="18" t="str">
+        <x:v>P02</x:v>
+      </x:c>
+      <x:c r="B101" s="18" t="str">
+        <x:v>low: 150
+high: 150</x:v>
+      </x:c>
+      <x:c r="C101" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="40" customHeight="1">
+      <x:c r="A102" s="18" t="str">
+        <x:v>L04</x:v>
+      </x:c>
+      <x:c r="B102" s="18" t="str">
+        <x:v>low: 15000
+high: 15000</x:v>
+      </x:c>
+      <x:c r="C102" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="40" customHeight="1">
+      <x:c r="A103" s="18" t="str">
+        <x:v>L05</x:v>
+      </x:c>
+      <x:c r="B103" s="18" t="str">
+        <x:v>low: 800
+high: 800</x:v>
+      </x:c>
+      <x:c r="C103" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="40" customHeight="1">
+      <x:c r="A104" s="18" t="str">
+        <x:v>L06</x:v>
+      </x:c>
+      <x:c r="B104" s="18" t="str">
+        <x:v>low: 10000
+high: 10000</x:v>
+      </x:c>
+      <x:c r="C104" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="40" customHeight="1">
+      <x:c r="A105" s="18" t="str">
+        <x:v>L07</x:v>
+      </x:c>
+      <x:c r="B105" s="18" t="str">
+        <x:v>low: 4000
+high: 4000</x:v>
+      </x:c>
+      <x:c r="C105" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="40" customHeight="1">
+      <x:c r="A106" s="18" t="str">
+        <x:v>L08</x:v>
+      </x:c>
+      <x:c r="B106" s="18" t="str">
+        <x:v>low: 300
+high: 300</x:v>
+      </x:c>
+      <x:c r="C106" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="40" customHeight="1">
+      <x:c r="A107" s="18" t="str">
+        <x:v>FUT01</x:v>
+      </x:c>
+      <x:c r="B107" s="18" t="str">
+        <x:v>low: 6000
+high: 6000</x:v>
+      </x:c>
+      <x:c r="C107" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="40" customHeight="1">
+      <x:c r="A108" s="18" t="str">
+        <x:v>FUT02</x:v>
+      </x:c>
+      <x:c r="B108" s="18" t="str">
+        <x:v>low: 500
+high: 500</x:v>
+      </x:c>
+      <x:c r="C108" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="40" customHeight="1">
+      <x:c r="A109" s="18" t="str">
+        <x:v>FUT03</x:v>
+      </x:c>
+      <x:c r="B109" s="18" t="str">
+        <x:v>low: 1000
+high: 1000</x:v>
+      </x:c>
+      <x:c r="C109" s="18" t="str">
+        <x:v>歷史來源欄位；採用 Purchase 的現行價格欄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="30" customHeight="1">
+      <x:c r="A110" s="25" t="str">
+        <x:v>PCB 補充來源</x:v>
+      </x:c>
+      <x:c r="B110" s="25" t="str"/>
+      <x:c r="C110" s="25" t="str"/>
+    </x:row>
+    <x:row r="111" ht="222" customHeight="1">
+      <x:c r="A111" s="18" t="str">
+        <x:v>1: C1</x:v>
+      </x:c>
+      <x:c r="B111" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 1
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C1","purpose_zh":"U2 OUT 系統供電節點至 GND 的去耦／緩衝電容。","purpose_en":"Decoupling/buffering between the U2 OUT system-supply node and ground.","location_zh":"原理圖第 1 頁：充電／電源路徑","location_en":"Schematic page 1: charger / power path","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填容值。","spec_en":"No capacitance is given in the vendor BOM or schematic.","purpose_zh":"C1: U2 OUT 系統供電節點至 GND 的去耦／緩衝電容。","purpose_en":"C1: Decoupling/buffering between the U2 OUT system-supply node and ground.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 1</x:v>
+      </x:c>
+      <x:c r="C111" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="222" customHeight="1">
+      <x:c r="A112" s="18" t="str">
+        <x:v>2: C2</x:v>
+      </x:c>
+      <x:c r="B112" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 2
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C2","purpose_zh":"U1 Vin 升壓輸入節點至 GND 的去耦電容。","purpose_en":"Input decoupling from the U1 boost-input node to ground.","location_zh":"原理圖第 1 頁：升壓電源","location_en":"Schematic page 1: boost supply","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填容值。","spec_en":"No capacitance is given in the vendor BOM or schematic.","purpose_zh":"C2: U1 Vin 升壓輸入節點至 GND 的去耦電容。","purpose_en":"C2: Input decoupling from the U1 boost-input node to ground.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 2</x:v>
+      </x:c>
+      <x:c r="C112" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="250" customHeight="1">
+      <x:c r="A113" s="18" t="str">
+        <x:v>3: C3</x:v>
+      </x:c>
+      <x:c r="B113" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 3
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C3","purpose_zh":"U1 輸出、標為 5V 的節點至 GND 的濾波电容；實際設定仍取決於未提供的 R6/R8。","purpose_en":"Output filtering on the net labelled 5V; the actual setting still depends on unspecified R6/R8.","location_zh":"原理圖第 1 頁：升壓電源","location_en":"Schematic page 1: boost supply","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填容值。","spec_en":"No capacitance is given in the vendor BOM or schematic.","purpose_zh":"C3: U1 輸出、標為 5V 的節點至 GND 的濾波电容；實際設定仍取決於未提供的 R6/R8。","purpose_en":"C3: Output filtering on the net labelled 5V; the actual setting still depends on unspecified R6/R8.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 3</x:v>
+      </x:c>
+      <x:c r="C113" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="250" customHeight="1">
+      <x:c r="A114" s="18" t="str">
+        <x:v>4: C4</x:v>
+      </x:c>
+      <x:c r="B114" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 4
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C4","purpose_zh":"U1 輸出、標為 5V 的節點至 GND 的濾波电容；實際設定仍取決於未提供的 R6/R8。","purpose_en":"Output filtering on the net labelled 5V; the actual setting still depends on unspecified R6/R8.","location_zh":"原理圖第 1 頁：升壓電源","location_en":"Schematic page 1: boost supply","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填容值。","spec_en":"No capacitance is given in the vendor BOM or schematic.","purpose_zh":"C4: U1 輸出、標為 5V 的節點至 GND 的濾波电容；實際設定仍取決於未提供的 R6/R8。","purpose_en":"C4: Output filtering on the net labelled 5V; the actual setting still depends on unspecified R6/R8.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 4</x:v>
+      </x:c>
+      <x:c r="C114" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="250" customHeight="1">
+      <x:c r="A115" s="18" t="str">
+        <x:v>5: C5</x:v>
+      </x:c>
+      <x:c r="B115" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 5
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C5","purpose_zh":"U1 輸出、標為 5V 的節點至 GND 的濾波电容；實際設定仍取決於未提供的 R6/R8。","purpose_en":"Output filtering on the net labelled 5V; the actual setting still depends on unspecified R6/R8.","location_zh":"原理圖第 1 頁：升壓電源","location_en":"Schematic page 1: boost supply","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填容值。","spec_en":"No capacitance is given in the vendor BOM or schematic.","purpose_zh":"C5: U1 輸出、標為 5V 的節點至 GND 的濾波电容；實際設定仍取決於未提供的 R6/R8。","purpose_en":"C5: Output filtering on the net labelled 5V; the actual setting still depends on unspecified R6/R8.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 5</x:v>
+      </x:c>
+      <x:c r="C115" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="222" customHeight="1">
+      <x:c r="A116" s="18" t="str">
+        <x:v>6: C6</x:v>
+      </x:c>
+      <x:c r="B116" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 6
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C6","purpose_zh":"USB 5V_USB 至 GND 的輸入去耦電容。","purpose_en":"Input decoupling from USB 5V_USB to ground.","location_zh":"原理圖第 1 頁：USB／充電輸入","location_en":"Schematic page 1: USB / charger input","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填容值。","spec_en":"No capacitance is given in the vendor BOM or schematic.","purpose_zh":"C6: USB 5V_USB 至 GND 的輸入去耦電容。","purpose_en":"C6: Input decoupling from USB 5V_USB to ground.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 6</x:v>
+      </x:c>
+      <x:c r="C116" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="236" customHeight="1">
+      <x:c r="A117" s="18" t="str">
+        <x:v>7: C7</x:v>
+      </x:c>
+      <x:c r="B117" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 7
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C7","purpose_zh":"U3 P1 供電節點至 GND 的去耦電容；U3 型號未提供。","purpose_en":"Decoupling from the U3 P1 supply node to ground; U3 is unidentified.","location_zh":"原理圖第 1 頁：U3 電源控制周邊","location_en":"Schematic page 1: U3 power-control circuitry","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填容值。","spec_en":"No capacitance is given in the vendor BOM or schematic.","purpose_zh":"C7: U3 P1 供電節點至 GND 的去耦電容；U3 型號未提供。","purpose_en":"C7: Decoupling from the U3 P1 supply node to ground; U3 is unidentified.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 7</x:v>
+      </x:c>
+      <x:c r="C117" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="222" customHeight="1">
+      <x:c r="A118" s="18" t="str">
+        <x:v>8: C8</x:v>
+      </x:c>
+      <x:c r="B118" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 8
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C8","purpose_zh":"U2 BAT／J1 電池正端節點至 GND 的電容。","purpose_en":"Capacitor from the U2 BAT / J1 battery-positive node to ground.","location_zh":"原理圖第 1 頁：電池／充電","location_en":"Schematic page 1: battery / charger","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填容值。","spec_en":"No capacitance is given in the vendor BOM or schematic.","purpose_zh":"C8: U2 BAT／J1 電池正端節點至 GND 的電容。","purpose_en":"C8: Capacitor from the U2 BAT / J1 battery-positive node to ground.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 8</x:v>
+      </x:c>
+      <x:c r="C118" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="250" customHeight="1">
+      <x:c r="A119" s="18" t="str">
+        <x:v>9: C9</x:v>
+      </x:c>
+      <x:c r="B119" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 9
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C9","purpose_zh":"R10/R12 分壓中點、U3 P2 至 GND 的濾波電容；具體控制功能待 U3 型號確認。","purpose_en":"Filtering from the R10/R12 divider midpoint / U3 P2 to ground; control function requires the U3 identity.","location_zh":"原理圖第 1 頁：U3 電源控制周邊","location_en":"Schematic page 1: U3 power-control circuitry","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填容值。","spec_en":"No capacitance is given in the vendor BOM or schematic.","purpose_zh":"C9: R10/R12 分壓中點、U3 P2 至 GND 的濾波電容；具體控制功能待 U3 型號確認。","purpose_en":"C9: Filtering from the R10/R12 divider midpoint / U3 P2 to ground; control function requires the U3 identity.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 9</x:v>
+      </x:c>
+      <x:c r="C119" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="250" customHeight="1">
+      <x:c r="A120" s="18" t="str">
+        <x:v>10: C10</x:v>
+      </x:c>
+      <x:c r="B120" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 10
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C10","purpose_zh":"U3 P6 至 GND；U3 型號未提供，不能確定其定時／補償等具體功能。","purpose_en":"Connected from U3 P6 to ground; timing/compensation or other function cannot be assigned without its identity.","location_zh":"原理圖第 1 頁：U3 電源控制周邊","location_en":"Schematic page 1: U3 power-control circuitry","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填容值。","spec_en":"No capacitance is given in the vendor BOM or schematic.","purpose_zh":"C10: U3 P6 至 GND；U3 型號未提供，不能確定其定時／補償等具體功能。","purpose_en":"C10: Connected from U3 P6 to ground; timing/compensation or other function cannot be assigned without its identity.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 10</x:v>
+      </x:c>
+      <x:c r="C120" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="250" customHeight="1">
+      <x:c r="A121" s="18" t="str">
+        <x:v>11: C11</x:v>
+      </x:c>
+      <x:c r="B121" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 11
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C11","purpose_zh":"U3 P4 至 GND；U3 型號未提供，不能確定其定時／補償等具體功能。","purpose_en":"Connected from U3 P4 to ground; timing/compensation or other function cannot be assigned without its identity.","location_zh":"原理圖第 1 頁：U3 電源控制周邊","location_en":"Schematic page 1: U3 power-control circuitry","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填容值。","spec_en":"No capacitance is given in the vendor BOM or schematic.","purpose_zh":"C11: U3 P4 至 GND；U3 型號未提供，不能確定其定時／補償等具體功能。","purpose_en":"C11: Connected from U3 P4 to ground; timing/compensation or other function cannot be assigned without its identity.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 11</x:v>
+      </x:c>
+      <x:c r="C121" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="222" customHeight="1">
+      <x:c r="A122" s="18" t="str">
+        <x:v>12: C12</x:v>
+      </x:c>
+      <x:c r="B122" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 15
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 12
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C12","purpose_zh":"LED 區 5V 至 GND 的局部儲能電容；原圖有極性符號。","purpose_en":"Local bulk capacitor between LED 5V and ground; the schematic uses a polarized symbol.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱容值 47uF。","spec_en":"Vendor nominal capacitance: 47uF.","purpose_zh":"C12: LED 區 5V 至 GND 的局部儲能電容；原圖有極性符號。","purpose_en":"C12: Local bulk capacitor between LED 5V and ground; the schematic uses a polarized symbol.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 12</x:v>
+      </x:c>
+      <x:c r="C122" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="236" customHeight="1">
+      <x:c r="A123" s="18" t="str">
+        <x:v>13: C13,C18</x:v>
+      </x:c>
+      <x:c r="B123" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 8
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 13
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C13","purpose_zh":"ESP32 3V3_DIG 供電去耦。","purpose_en":"ESP32 3V3_DIG supply decoupling.","location_zh":"原理圖第 2 頁：ESP32","location_en":"Schematic page 2: ESP32","page":2},{"reference":"C18","purpose_zh":"U5 的 3V3_DIG 輸出電容。","purpose_en":"U5 3V3_DIG output capacitor.","location_zh":"原理圖第 2 頁：3V3 LDO","location_en":"Schematic page 2: 3V3 LDO","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱容值 22uF。","spec_en":"Vendor nominal capacitance: 22uF.","purpose_zh":"C13: ESP32 3V3_DIG 供電去耦。；C18: U5 的 3V3_DIG 輸出電容。","purpose_en":"C13: ESP32 3V3_DIG supply decoupling.；C18: U5 3V3_DIG output capacitor.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 13</x:v>
+      </x:c>
+      <x:c r="C123" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="194" customHeight="1">
+      <x:c r="A124" s="18" t="str">
+        <x:v>14: C14,C15,C22,C25</x:v>
+      </x:c>
+      <x:c r="B124" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 14
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C14","purpose_zh":"ESP32 3V3_DIG 供電去耦。","purpose_en":"ESP32 3V3_DIG supply decoupling.","location_zh":"原理圖第 2 頁：ESP32","location_en":"Schematic page 2: ESP32","page":2},{"reference":"C15","purpose_zh":"跨接 SW2 的 ESP_EN 至 GND，屬復位／啟用節點電容。","purpose_en":"ESP_EN-to-ground capacitor across SW2 in the reset/enable network.","location_zh":"原理圖第 2 頁：ESP32 復位","location_en":"Schematic page 2: ESP32 reset","page":2},{"reference":"C22","purpose_zh":"U7 的 3V3_ANA 輸入去耦。","purpose_en":"U7 3V3_ANA input decoupling.","location_zh":"原理圖第 2 頁：2V5_REF","location_en":"Schematic page 2: 2V5_REF","page":2},{"reference":"C25","purpose_zh":"R31 後方 U8 局部供電至 GND 的電容，與 R31 構成供電濾波。C26 原圖有極性符號。","purpose_en":"Capacitors from the U8 local supply after R31 to ground, forming supply filtering with R31. C26 has a polarized</x:v>
+      </x:c>
+      <x:c r="C124" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="208" customHeight="1">
+      <x:c r="A125" s="18" t="str">
+        <x:v>14: C14,C15,C22,C25 （續）</x:v>
+      </x:c>
+      <x:c r="B125" s="18" t="str">
+        <x:v> symbol.","location_zh":"原理圖第 2 頁：TIA 供電","location_en":"Schematic page 2: TIA supply","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱容值 0.1uF。","spec_en":"Vendor nominal capacitance: 0.1uF.","purpose_zh":"C14: ESP32 3V3_DIG 供電去耦。；C15: 跨接 SW2 的 ESP_EN 至 GND，屬復位／啟用節點電容。；C22: U7 的 3V3_ANA 輸入去耦。；C25: R31 後方 U8 局部供電至 GND 的電容，與 R31 構成供電濾波。C26 原圖有極性符號。","purpose_en":"C14: ESP32 3V3_DIG supply decoupling.；C15: ESP_EN-to-ground capacitor across SW2 in the reset/enable network.；C22: U7 3V3_ANA input decoupling.；C25: Capacitors from the U8 local supply after R31 to ground, forming supply filtering with R31. C26 has a polarized symbol.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 14</x:v>
+      </x:c>
+      <x:c r="C125" s="18" t="str"/>
+    </x:row>
+    <x:row r="126" ht="194" customHeight="1">
+      <x:c r="A126" s="18" t="str">
+        <x:v>15: C16,C17,C23,C28</x:v>
+      </x:c>
+      <x:c r="B126" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 8
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 15
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C16","purpose_zh":"ESP_EN 至 GND，與 R15 構成啟用／復位 RC 網路。","purpose_en":"ESP_EN-to-ground capacitor forming the enable/reset RC network with R15.","location_zh":"原理圖第 2 頁：ESP32 復位","location_en":"Schematic page 2: ESP32 reset","page":2},{"reference":"C17","purpose_zh":"U5 的 5V 輸入去耦。","purpose_en":"U5 5V input decoupling.","location_zh":"原理圖第 2 頁：3V3 LDO","location_en":"Schematic page 2: 3V3 LDO","page":2},{"reference":"C23","purpose_zh":"U7 VREF_2V5 輸出電容。","purpose_en":"U7 VREF_2V5 output capacitor.","location_zh":"原理圖第 2 頁：2V5_REF","location_en":"Schematic page 2: 2V5_REF","page":2},{"reference":"C28","purpose_zh":"與 R34 串聯，形成 VREF_2V5 至 GND 的參考電壓旁路支路。","purpose_en":"In series with R34 in a VREF_2V5-to-ground reference-bypass</x:v>
+      </x:c>
+      <x:c r="C126" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="194" customHeight="1">
+      <x:c r="A127" s="18" t="str">
+        <x:v>15: C16,C17,C23,C28 （續）</x:v>
+      </x:c>
+      <x:c r="B127" s="18" t="str">
+        <x:v> branch.","location_zh":"原理圖第 2 頁：ADC 參考","location_en":"Schematic page 2: ADC reference","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱容值 10uF。","spec_en":"Vendor nominal capacitance: 10uF.","purpose_zh":"C16: ESP_EN 至 GND，與 R15 構成啟用／復位 RC 網路。；C17: U5 的 5V 輸入去耦。；C23: U7 VREF_2V5 輸出電容。；C28: 與 R34 串聯，形成 VREF_2V5 至 GND 的參考電壓旁路支路。","purpose_en":"C16: ESP_EN-to-ground capacitor forming the enable/reset RC network with R15.；C17: U5 5V input decoupling.；C23: U7 VREF_2V5 output capacitor.；C28: In series with R34 in a VREF_2V5-to-ground reference-bypass branch.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 15</x:v>
+      </x:c>
+      <x:c r="C127" s="18" t="str"/>
+    </x:row>
+    <x:row r="128" ht="166" customHeight="1">
+      <x:c r="A128" s="18" t="str">
+        <x:v>16: C19,C20,C27,C29</x:v>
+      </x:c>
+      <x:c r="B128" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 16
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C19","purpose_zh":"U6 的 5V 輸入去耦。","purpose_en":"U6 5V input decoupling.","location_zh":"原理圖第 2 頁：3V3 LDO","location_en":"Schematic page 2: 3V3 LDO","page":2},{"reference":"C20","purpose_zh":"U6 的 3V3_ANA 輸出電容。","purpose_en":"U6 3V3_ANA output capacitor.","location_zh":"原理圖第 2 頁：3V3 LDO","location_en":"Schematic page 2: 3V3 LDO","page":2},{"reference":"C27","purpose_zh":"U9 DVDD／3V3_DIG 供電去耦。","purpose_en":"U9 DVDD / 3V3_DIG decoupling.","location_zh":"原理圖第 2 頁：ADC","location_en":"Schematic page 2: ADC","page":2},{"reference":"C29","purpose_zh":"U9 AVDD／3V3_ANA 供電去耦。","purpose_en":"U9 AVDD / 3V3_ANA</x:v>
+      </x:c>
+      <x:c r="C128" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="152" customHeight="1">
+      <x:c r="A129" s="18" t="str">
+        <x:v>16: C19,C20,C27,C29 （續）</x:v>
+      </x:c>
+      <x:c r="B129" s="18" t="str">
+        <x:v> decoupling.","location_zh":"原理圖第 2 頁：ADC","location_en":"Schematic page 2: ADC","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱容值 1uF。","spec_en":"Vendor nominal capacitance: 1uF.","purpose_zh":"C19: U6 的 5V 輸入去耦。；C20: U6 的 3V3_ANA 輸出電容。；C27: U9 DVDD／3V3_DIG 供電去耦。；C29: U9 AVDD／3V3_ANA 供電去耦。","purpose_en":"C19: U6 5V input decoupling.；C20: U6 3V3_ANA output capacitor.；C27: U9 DVDD / 3V3_DIG decoupling.；C29: U9 AVDD / 3V3_ANA decoupling.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 16</x:v>
+      </x:c>
+      <x:c r="C129" s="18" t="str"/>
+    </x:row>
+    <x:row r="130" ht="278" customHeight="1">
+      <x:c r="A130" s="18" t="str">
+        <x:v>17: C21</x:v>
+      </x:c>
+      <x:c r="B130" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 17
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C21","purpose_zh":"與 R27 並聯，從 U8 輸出回授至反相輸入；影響跨阻放大器補償與頻寬。","purpose_en":"In parallel with R27 from U8 output to its inverting input; affects transimpedance compensation and bandwidth.","location_zh":"原理圖第 2 頁：TIA","location_en":"Schematic page 2: TIA","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱容值 2.2pF。","spec_en":"Vendor nominal capacitance: 2.2pF.","purpose_zh":"C21: 與 R27 並聯，從 U8 輸出回授至反相輸入；影響跨阻放大器補償與頻寬。","purpose_en":"C21: In parallel with R27 from U8 output to its inverting input; affects transimpedance compensation and bandwidth.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。 2.2 pF 為小訊號回授值，焊墊／走線寄生不可忽略；低漏電與合適介電材質須廠商選定。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks. At 2.2 pF, pad/trace parasitics matter; the vendor must select suitable low-leakage construction/dielectric."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 17</x:v>
+      </x:c>
+      <x:c r="C130" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="236" customHeight="1">
+      <x:c r="A131" s="18" t="str">
+        <x:v>18: C24</x:v>
+      </x:c>
+      <x:c r="B131" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 18
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C24","purpose_zh":"跨 ADC_AINP 與 ADC_AINN，與 R29/R36 形成 ADC 輸入濾波網路。","purpose_en":"Across ADC_AINP and ADC_AINN, part of the ADC-input filtering network with R29/R36.","location_zh":"原理圖第 2 頁：TIA／ADC","location_en":"Schematic page 2: TIA / ADC","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱容值 1000pF。","spec_en":"Vendor nominal capacitance: 1000pF.","purpose_zh":"C24: 跨 ADC_AINP 與 ADC_AINN，與 R29/R36 形成 ADC 輸入濾波網路。","purpose_en":"C24: Across ADC_AINP and ADC_AINN, part of the ADC-input filtering network with R29/R36.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 18</x:v>
+      </x:c>
+      <x:c r="C131" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="250" customHeight="1">
+      <x:c r="A132" s="18" t="str">
+        <x:v>19: C26</x:v>
+      </x:c>
+      <x:c r="B132" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 15
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 19
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"C26","purpose_zh":"R31 後方 U8 局部供電至 GND 的電容，與 R31 構成供電濾波。C26 原圖有極性符號。","purpose_en":"Capacitors from the U8 local supply after R31 to ground, forming supply filtering with R31. C26 has a polarized symbol.","location_zh":"原理圖第 2 頁：TIA 供電","location_en":"Schematic page 2: TIA supply","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱容值 100uF。","spec_en":"Vendor nominal capacitance: 100uF.","purpose_zh":"C26: R31 後方 U8 局部供電至 GND 的電容，與 R31 構成供電濾波。C26 原圖有極性符號。","purpose_en":"C26: Capacitors from the U8 local supply after R31 to ground, forming supply filtering with R31. C26 has a polarized symbol.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、耐壓、容差、介電材質／型式尚未提供；電源電容需另核對有效容值、ESR 與穩定性要求。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, voltage rating, tolerance and dielectric/type are not supplied; power capacitors also require effective-capacitance, ESR and stability checks."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 19</x:v>
+      </x:c>
+      <x:c r="C132" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="180" customHeight="1">
+      <x:c r="A133" s="18" t="str">
+        <x:v>20: DPS1,DPS2</x:v>
+      </x:c>
+      <x:c r="B133" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 2
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 20
+source_ids: ["vendor_BOM","schematic"]
+per_reference: []
+orderability: incomplete_component_specification
+details: {"spec_zh":"僅標示 LED；共 2 顆。","spec_en":"Only identified as LED; two devices.","purpose_zh":"DPS1 接 U2 PGOOD、配 R5；DPS2 接 U2 CHG、配 R7，顯示電源／充電狀態。","purpose_en":"DPS1 is connected to U2 PGOOD via R5; DPS2 to U2 CHG via R7 for power/charging status.","missing_zh":"顏色、廠牌／MPN、封裝尺寸／高度、順向電壓／電流與亮度均未提供。","missing_en":"Color, manufacturer/MPN, package size/height, forward voltage/current and brightness are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 20</x:v>
+      </x:c>
+      <x:c r="C133" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="236" customHeight="1">
+      <x:c r="A134" s="18" t="str">
+        <x:v>21: D1,D2,D3,D4</x:v>
+      </x:c>
+      <x:c r="B134" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 17
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 21
+source_ids: ["vendor_BOM","schematic","WURTH_LED"]
+per_reference: []
+orderability: identified_part_pending_assembly_verification
+details: {"spec_zh":"Würth Elektronik 155124BS73200；1204 側發光 SMD；資料表在 20 mA 下典型峰值 468 nm／主波長 470 nm、視角 120°。","spec_en":"Würth Elektronik 155124BS73200; 1204 side-view SMD; datasheet at 20 mA gives typical peak 468 nm / dominant wavelength 470 nm and 120° viewing angle.","purpose_zh":"D1–D4 由 Q1–Q4 低側開關調變；各有 100 Ω 串聯電阻。GPIO25/26/27/32 對應 LED1/2/3/4。","purpose_en":"D1–D4 are modulated by low-side switches Q1–Q4 with individual 100 Ω series resistors. GPIO25/26/27/32 map to LED1/2/3/4.","missing_zh":"須核對實際焊接方向／高度、光學軸與 well 對位、實際電流及光功率；20 mA 是資料表測試條件，非已驗證板上電流。","missing_en":"Verify assembled orientation/height, optical-axis alignment to wells, operating current and optical power; 20 mA is a datasheet test condition, not a verified board current."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 21</x:v>
+      </x:c>
+      <x:c r="C134" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="236" customHeight="1">
+      <x:c r="A135" s="18" t="str">
+        <x:v>22: D5</x:v>
+      </x:c>
+      <x:c r="B135" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 68
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 22
+source_ids: ["vendor_BOM","schematic","VISHAY_PD"]
+per_reference: []
+orderability: identified_part_pending_assembly_verification
+details: {"spec_zh":"Vishay VEMD5060X01；頂視 SMD，外形 5×4×0.9 mm；感光面積 7.5 mm²；可見光至近紅外感測。","spec_en":"Vishay VEMD5060X01; top-view SMD, 5×4×0.9 mm body; 7.5 mm² photosensitive area; visible-to-near-infrared response.","purpose_zh":"D5 是四井共用 PD；陰極連 PD_SUM／U8 反相輸入，陽極接 GND。藍光與綠光皆可被接收，必須搭配光學濾波與空白校正。","purpose_en":"D5 is the single PD shared by four wells; cathode to PD_SUM / U8 inverting input and anode to ground. It detects both blue and green light, requiring optical filtering and blank correction.","missing_zh":"實際感光區中心與封裝中心不可混同；裝配座標、濾片／墊圈遮擋與角度接受度须核對。廠商需確認最終訂購後綴及來料。","missing_en":"Do not equate the active-area center with the package center; verify assembly coordinates, filter/gasket obscuration and angular acceptance. Confirm final order suffix and supplied part."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 22</x:v>
+      </x:c>
+      <x:c r="C135" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="180" customHeight="1">
+      <x:c r="A136" s="18" t="str">
+        <x:v>23: FD1,FD2,FD3,FD4,FD5,FD6,FD
+7,FD8</x:v>
+      </x:c>
+      <x:c r="B136" s="18" t="str">
+        <x:v>status: PCB fiducial，不是採購元件
+unit_price: 0
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 23
+source_ids: ["vendor_BOM","schematic"]
+per_reference: []
+orderability: PCB_feature_not_separate_purchase
+details: {"spec_zh":"FD_040；8 個定位標記。","spec_en":"FD_040; eight fiducials.","purpose_zh":"供 SMT 視覺定位，不是額外焊接的 LED 或感測器。","purpose_en":"Provide vision alignment for SMT assembly; these are not separate LEDs or sensors.","missing_zh":"銅面／阻焊開窗與定位尺寸由製板資料確認；不另購零件。","missing_en":"Confirm copper/solder-mask geometry in fabrication data; do not purchase separate components."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 23</x:v>
+      </x:c>
+      <x:c r="C136" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="194" customHeight="1">
+      <x:c r="A137" s="18" t="str">
+        <x:v>24: H1,H2,H3,H4</x:v>
+      </x:c>
+      <x:c r="B137" s="18" t="str">
+        <x:v>status: PCB孔位，不另當电子零件買
+unit_price: 0
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 24
+source_ids: ["vendor_BOM","schematic"]
+per_reference: []
+orderability: PCB_feature_not_separate_purchase
+details: {"spec_zh":"H1–H4；原廠標示 CON(銅柱孔)。","spec_en":"H1–H4; vendor label CON (standoff holes).","purpose_zh":"PCB 機械固定孔，不是電子連接器；額外螺絲／螺帽見其他材料表，勿重複計價。","purpose_en":"Mechanical PCB fixing holes, not electrical connectors; screws/nuts are listed in the separate materials BOM and must not be counted twice.","missing_zh":"孔徑、鍍孔／非鍍孔、銅箔避讓與裝配間隙須依製板圖／實板確認；本列未指定螺絲尺寸。","missing_en":"Verify diameter, plated/non-plated status, copper keepout and clearance from fabrication drawings/board; this row does not specify a screw size."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 24</x:v>
+      </x:c>
+      <x:c r="C137" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="222" customHeight="1">
+      <x:c r="A138" s="18" t="str">
+        <x:v>25: J1</x:v>
+      </x:c>
+      <x:c r="B138" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 30
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 25
+source_ids: ["vendor_BOM","schematic","TI_BQ24074"]
+per_reference: []
+orderability: incomplete_component_specification
+details: {"spec_zh":"原廠僅標 Battery_Case；原圖腳1接 BAT，腳2接 GND。","spec_en":"Only Battery_Case is specified; schematic pin 1 connects to BAT and pin 2 to ground.","purpose_zh":"接 U2 BQ24074 單節鋰離子／鋰聚合物 4.2 V 充電架構；不能由此推定為 18650 電池座。","purpose_en":"Connects to the BQ24074 single-cell Li-ion/Li-poly 4.2 V charging architecture; this does not establish an 18650 holder.","missing_zh":"完整MPN、電池尺寸／化學與保護配置、極性標記、安裝孔與含電池高度、額定電流未完整提供；R1–R3/R9 亦未定，先請廠商確認。","missing_en":"MPN, cell size/chemistry/protection, polarity marking, mounting and height with cell, and current rating are incomplete; R1–R3/R9 are also unspecified. Obtain vendor confirmation first."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 25</x:v>
+      </x:c>
+      <x:c r="C138" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="208" customHeight="1">
+      <x:c r="A139" s="18" t="str">
+        <x:v>26: J2</x:v>
+      </x:c>
+      <x:c r="B139" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 20
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 26
+source_ids: ["vendor_BOM","schematic"]
+per_reference: []
+orderability: incomplete_component_specification
+details: {"spec_zh":"VBUS 接 5V_USB；CC1/CC2 經 R13/R14 至 GND；資料線 D+/D− 與 SBU 未接。","spec_en":"VBUS connects to 5V_USB; CC1/CC2 connect through R13/R14 to ground; D+/D− and SBU are unconnected.","purpose_zh":"提供電源／充電輸入，不能用此孔作原生 USB 韌體燒錄或資料傳输；J3 是 UART 介面。","purpose_en":"Power/charging input, not a native USB programming/data port; J3 provides the UART interface.","missing_zh":"完整MPN、封裝與固定腳、孔口位置／高度、額定電流未給；R13/R14 數值未給，USB-C 供電配置待確認。","missing_en":"MPN, footprint/retention tabs, opening location/height and current rating are absent; R13/R14 values are absent, so confirm USB-C power configuration."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 26</x:v>
+      </x:c>
+      <x:c r="C139" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="208" customHeight="1">
+      <x:c r="A140" s="18" t="str">
+        <x:v>27: J3</x:v>
+      </x:c>
+      <x:c r="B140" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 5
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 27
+source_ids: ["vendor_BOM","schematic"]
+per_reference: []
+orderability: incomplete_component_specification
+details: {"spec_zh":"原圖腳1=3V3_DIG、2=ESP32 TXD0、3=ESP32 RXD0、4=GND。","spec_en":"Schematic pin 1=3V3_DIG, 2=ESP32 TXD0, 3=ESP32 RXD0, 4=GND.","purpose_zh":"ESP32 3.3 V UART 燒錄／除錯介面；連接轉接器時 TX/RX 交叉且核對供電，不能將5 V邏輯直接接入。","purpose_en":"ESP32 3.3 V UART programming/debug interface; cross TX/RX and verify power wiring. Do not apply 5 V logic directly.","missing_zh":"廠牌／MPN、針距、直角／直立、針長與高度、對接線材未提供；不能自動假定2.54 mm。","missing_en":"Manufacturer/MPN, pitch, straight/right-angle form, pin length/height and mating cable are unspecified; do not automatically assume 2.54 mm."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 27</x:v>
+      </x:c>
+      <x:c r="C140" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="180" customHeight="1">
+      <x:c r="A141" s="18" t="str">
+        <x:v>28: L1</x:v>
+      </x:c>
+      <x:c r="B141" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 10
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 28
+source_ids: ["vendor_BOM","schematic","TI_TPS61023"]
+per_reference: []
+orderability: incomplete_component_specification
+details: {"spec_zh":"L1；原廠無電感值／MPN。","spec_en":"L1; inductance and MPN are absent.","purpose_zh":"跨 U1 Vin 與 SW，為 TPS61023 升壓能量儲存元件。","purpose_en":"Between U1 Vin and SW; the TPS61023 boost energy-storage element.","missing_zh":"電感值、飽和／RMS 電流、DCR、屏蔽型式、封裝／高度與完整MPN皆待廠商確認。","missing_en":"Inductance, saturation/RMS current, DCR, shielding, package/height and orderable MPN all require vendor confirmation."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 28</x:v>
+      </x:c>
+      <x:c r="C141" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="208" customHeight="1">
+      <x:c r="A142" s="18" t="str">
+        <x:v>29: Q1,Q2,Q3,Q4</x:v>
+      </x:c>
+      <x:c r="B142" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 5
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 29
+source_ids: ["vendor_BOM","schematic","AOS_AO3400A"]
+per_reference: []
+orderability: identified_part_pending_assembly_verification
+details: {"spec_zh":"AOS AO3400A；30 V N-MOSFET，SOT-23；資料表提供低閘極電壓導通規格。","spec_en":"AOS AO3400A; 30 V N-channel MOSFET, SOT-23; low-gate-voltage on-resistance is specified.","purpose_zh":"Q1–Q4 分別作 D1–D4 LED 低側開關；由各 LED_GATE 經串聯電阻驅動，閘極有下拉。","purpose_en":"Q1–Q4 are low-side switches for LEDs D1–D4, driven by LED_GATE through series resistors with gate pull-downs.","missing_zh":"須核對封裝焊盤／腳位、來料及實際 LED 電流／溫升；器件最大額定值不等於板上允許負載。","missing_en":"Verify footprint/pinout, supplied part and operating LED current/temperature; device maximum ratings are not allowable board-load guarantees."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 29</x:v>
+      </x:c>
+      <x:c r="C142" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="222" customHeight="1">
+      <x:c r="A143" s="18" t="str">
+        <x:v>30: R1</x:v>
+      </x:c>
+      <x:c r="B143" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 30
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R1","purpose_zh":"U2 ITERM 至 GND，設定充電終止電流。","purpose_en":"U2 ITERM-to-ground resistor setting charge-termination current.","location_zh":"原理圖第 1 頁：充電／電源路徑","location_en":"Schematic page 1: charger / power path","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R1: U2 ITERM 至 GND，設定充電終止電流。","purpose_en":"R1: U2 ITERM-to-ground resistor setting charge-termination current.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 30</x:v>
+      </x:c>
+      <x:c r="C143" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="208" customHeight="1">
+      <x:c r="A144" s="18" t="str">
+        <x:v>31: R2</x:v>
+      </x:c>
+      <x:c r="B144" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 31
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R2","purpose_zh":"U2 ILIM 至 GND，設定輸入電流限制。","purpose_en":"U2 ILIM-to-ground resistor setting the input-current limit.","location_zh":"原理圖第 1 頁：充電／電源路徑","location_en":"Schematic page 1: charger / power path","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R2: U2 ILIM 至 GND，設定輸入電流限制。","purpose_en":"R2: U2 ILIM-to-ground resistor setting the input-current limit.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 31</x:v>
+      </x:c>
+      <x:c r="C144" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="208" customHeight="1">
+      <x:c r="A145" s="18" t="str">
+        <x:v>32: R3</x:v>
+      </x:c>
+      <x:c r="B145" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 32
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R3","purpose_zh":"U2 ISET 至 GND，設定充電電流。","purpose_en":"U2 ISET-to-ground resistor setting charge current.","location_zh":"原理圖第 1 頁：充電／電源路徑","location_en":"Schematic page 1: charger / power path","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R3: U2 ISET 至 GND，設定充電電流。","purpose_en":"R3: U2 ISET-to-ground resistor setting charge current.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 32</x:v>
+      </x:c>
+      <x:c r="C145" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="208" customHeight="1">
+      <x:c r="A146" s="18" t="str">
+        <x:v>33: R4</x:v>
+      </x:c>
+      <x:c r="B146" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 33
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R4","purpose_zh":"SW1 至 U1 EN／U3 P3 節點的串聯電阻。","purpose_en":"Series resistor from SW1 to the U1 EN / U3 P3 node.","location_zh":"原理圖第 1 頁：電源啟用","location_en":"Schematic page 1: power enable","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R4: SW1 至 U1 EN／U3 P3 節點的串聯電阻。","purpose_en":"R4: Series resistor from SW1 to the U1 EN / U3 P3 node.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 33</x:v>
+      </x:c>
+      <x:c r="C146" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="208" customHeight="1">
+      <x:c r="A147" s="18" t="str">
+        <x:v>34: R5</x:v>
+      </x:c>
+      <x:c r="B147" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 34
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R5","purpose_zh":"DPS1 狀態 LED 的串聯限流電阻。","purpose_en":"Series current-limiting resistor for the DPS1 status LED.","location_zh":"原理圖第 1 頁：充電狀態顯示","location_en":"Schematic page 1: charger status","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R5: DPS1 狀態 LED 的串聯限流電阻。","purpose_en":"R5: Series current-limiting resistor for the DPS1 status LED.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 34</x:v>
+      </x:c>
+      <x:c r="C147" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="222" customHeight="1">
+      <x:c r="A148" s="18" t="str">
+        <x:v>35: R6</x:v>
+      </x:c>
+      <x:c r="B148" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 35
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R6","purpose_zh":"5V 輸出至 U1 FB 的上臂回授電阻；與 R8 決定輸出設定。","purpose_en":"Upper feedback resistor from the 5V output to U1 FB; sets output together with R8.","location_zh":"原理圖第 1 頁：升壓電源","location_en":"Schematic page 1: boost supply","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R6: 5V 輸出至 U1 FB 的上臂回授電阻；與 R8 決定輸出設定。","purpose_en":"R6: Upper feedback resistor from the 5V output to U1 FB; sets output together with R8.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 35</x:v>
+      </x:c>
+      <x:c r="C148" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="208" customHeight="1">
+      <x:c r="A149" s="18" t="str">
+        <x:v>36: R7</x:v>
+      </x:c>
+      <x:c r="B149" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 36
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R7","purpose_zh":"DPS2 充電 LED 的串聯限流電阻。","purpose_en":"Series current-limiting resistor for the DPS2 charging LED.","location_zh":"原理圖第 1 頁：充電狀態顯示","location_en":"Schematic page 1: charger status","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R7: DPS2 充電 LED 的串聯限流電阻。","purpose_en":"R7: Series current-limiting resistor for the DPS2 charging LED.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 36</x:v>
+      </x:c>
+      <x:c r="C149" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="222" customHeight="1">
+      <x:c r="A150" s="18" t="str">
+        <x:v>37: R8</x:v>
+      </x:c>
+      <x:c r="B150" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 37
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R8","purpose_zh":"U1 FB 至 GND 的下臂回授電阻；與 R6 決定輸出設定。","purpose_en":"Lower feedback resistor from U1 FB to ground; sets output together with R6.","location_zh":"原理圖第 1 頁：升壓電源","location_en":"Schematic page 1: boost supply","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R8: U1 FB 至 GND 的下臂回授電阻；與 R6 決定輸出設定。","purpose_en":"R8: Lower feedback resistor from U1 FB to ground; sets output together with R6.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 37</x:v>
+      </x:c>
+      <x:c r="C150" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="236" customHeight="1">
+      <x:c r="A151" s="18" t="str">
+        <x:v>38: R9</x:v>
+      </x:c>
+      <x:c r="B151" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 38
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R9","purpose_zh":"U2 TS 至 GND 的偏壓支路；圖中僅畫電阻，不能宣稱已接電池溫度感測器。","purpose_en":"Bias branch from U2 TS to ground; the drawing only shows a resistor, not a verified battery-temperature sensor.","location_zh":"原理圖第 1 頁：充電 TS","location_en":"Schematic page 1: charger TS","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R9: U2 TS 至 GND 的偏壓支路；圖中僅畫電阻，不能宣稱已接電池溫度感測器。","purpose_en":"R9: Bias branch from U2 TS to ground; the drawing only shows a resistor, not a verified battery-temperature sensor.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 38</x:v>
+      </x:c>
+      <x:c r="C151" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="236" customHeight="1">
+      <x:c r="A152" s="18" t="str">
+        <x:v>39: R10</x:v>
+      </x:c>
+      <x:c r="B152" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 39
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R10","purpose_zh":"系統供電至 U3 P2 的分壓上臂，與 R12/C9 配合；U3 的確切功能未知。","purpose_en":"Upper divider from system supply to U3 P2, used with R12/C9; exact U3 function is unknown.","location_zh":"原理圖第 1 頁：U3 電源控制周邊","location_en":"Schematic page 1: U3 power-control circuitry","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R10: 系統供電至 U3 P2 的分壓上臂，與 R12/C9 配合；U3 的確切功能未知。","purpose_en":"R10: Upper divider from system supply to U3 P2, used with R12/C9; exact U3 function is unknown.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 39</x:v>
+      </x:c>
+      <x:c r="C152" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="208" customHeight="1">
+      <x:c r="A153" s="18" t="str">
+        <x:v>40: R11</x:v>
+      </x:c>
+      <x:c r="B153" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 40
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R11","purpose_zh":"U1 EN／U3 P3 共用節點至 GND 的下拉。","purpose_en":"Pull-down from the common U1 EN / U3 P3 node to ground.","location_zh":"原理圖第 1 頁：電源啟用","location_en":"Schematic page 1: power enable","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R11: U1 EN／U3 P3 共用節點至 GND 的下拉。","purpose_en":"R11: Pull-down from the common U1 EN / U3 P3 node to ground.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 40</x:v>
+      </x:c>
+      <x:c r="C153" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="236" customHeight="1">
+      <x:c r="A154" s="18" t="str">
+        <x:v>41: R12</x:v>
+      </x:c>
+      <x:c r="B154" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 41
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R12","purpose_zh":"U3 P2 至 GND 的分壓下臂，與 R10/C9 配合；U3 的確切功能未知。","purpose_en":"Lower divider from U3 P2 to ground, used with R10/C9; exact U3 function is unknown.","location_zh":"原理圖第 1 頁：U3 電源控制周邊","location_en":"Schematic page 1: U3 power-control circuitry","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R12: U3 P2 至 GND 的分壓下臂，與 R10/C9 配合；U3 的確切功能未知。","purpose_en":"R12: Lower divider from U3 P2 to ground, used with R10/C9; exact U3 function is unknown.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 41</x:v>
+      </x:c>
+      <x:c r="C154" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="236" customHeight="1">
+      <x:c r="A155" s="18" t="str">
+        <x:v>42: R13</x:v>
+      </x:c>
+      <x:c r="B155" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 42
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R13","purpose_zh":"USB-C CC1 至 GND 的下拉電阻。數值未給，不能自行填入典型值。","purpose_en":"USB-C CC1-to-ground pull-down; value is absent and must not be replaced by an assumed typical value.","location_zh":"原理圖第 1 頁：USB-C","location_en":"Schematic page 1: USB-C","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R13: USB-C CC1 至 GND 的下拉電阻。數值未給，不能自行填入典型值。","purpose_en":"R13: USB-C CC1-to-ground pull-down; value is absent and must not be replaced by an assumed typical value.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 42</x:v>
+      </x:c>
+      <x:c r="C155" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="236" customHeight="1">
+      <x:c r="A156" s="18" t="str">
+        <x:v>43: R14</x:v>
+      </x:c>
+      <x:c r="B156" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 43
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R14","purpose_zh":"USB-C CC2 至 GND 的下拉電阻。數值未給，不能自行填入典型值。","purpose_en":"USB-C CC2-to-ground pull-down; value is absent and must not be replaced by an assumed typical value.","location_zh":"原理圖第 1 頁：USB-C","location_en":"Schematic page 1: USB-C","page":1}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠 BOM 與原理圖皆未填阻值。","spec_en":"No resistance is given in the vendor BOM or schematic.","purpose_zh":"R14: USB-C CC2 至 GND 的下拉電阻。數值未給，不能自行填入典型值。","purpose_en":"R14: USB-C CC2-to-ground pull-down; value is absent and must not be replaced by an assumed typical value.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 43</x:v>
+      </x:c>
+      <x:c r="C156" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="166" customHeight="1">
+      <x:c r="A157" s="18" t="str">
+        <x:v>44: R15,R28,R35</x:v>
+      </x:c>
+      <x:c r="B157" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 44
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R15","purpose_zh":"ESP_EN 至 3V3_DIG 的上拉。","purpose_en":"Pull-up from ESP_EN to 3V3_DIG.","location_zh":"原理圖第 2 頁：ESP32 復位","location_en":"Schematic page 2: ESP32 reset","page":2},{"reference":"R28","purpose_zh":"U7 SHDN 至 Vin／3V3_ANA 的上拉。","purpose_en":"Pull-up from U7 SHDN to Vin / 3V3_ANA.","location_zh":"原理圖第 2 頁：2V5_REF","location_en":"Schematic page 2: 2V5_REF","page":2},{"reference":"R35","purpose_zh":"U9 DIN 至 3V3_DIG 的上拉，用於原圖標示的三線 CS 模式設定。","purpose_en":"DIN-to-3V3_DIG pull-up for the three-wire CS-mode configuration labelled in the schematic.","location_zh":"原理圖第 2</x:v>
+      </x:c>
+      <x:c r="C157" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="152" customHeight="1">
+      <x:c r="A158" s="18" t="str">
+        <x:v>44: R15,R28,R35 （續）</x:v>
+      </x:c>
+      <x:c r="B158" s="18" t="str">
+        <x:v> 頁：ADC","location_en":"Schematic page 2: ADC","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱阻值 10k。","spec_en":"Vendor nominal resistance: 10k.","purpose_zh":"R15: ESP_EN 至 3V3_DIG 的上拉。；R28: U7 SHDN 至 Vin／3V3_ANA 的上拉。；R35: U9 DIN 至 3V3_DIG 的上拉，用於原圖標示的三線 CS 模式設定。","purpose_en":"R15: Pull-up from ESP_EN to 3V3_DIG.；R28: Pull-up from U7 SHDN to Vin / 3V3_ANA.；R35: DIN-to-3V3_DIG pull-up for the three-wire CS-mode configuration labelled in the schematic.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 44</x:v>
+      </x:c>
+      <x:c r="C158" s="18" t="str"/>
+    </x:row>
+    <x:row r="159" ht="264" customHeight="1">
+      <x:c r="A159" s="18" t="str">
+        <x:v>45: R16,R21,R24,R29,R30,R31,R3
+6</x:v>
+      </x:c>
+      <x:c r="B159" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 45
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R16","purpose_zh":"D1 藍光 LED 的 5V 串聯限流電阻。","purpose_en":"5V series current-limiting resistor for blue LED D1.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2},{"reference":"R21","purpose_zh":"D2 藍光 LED 的 5V 串聯限流電阻。","purpose_en":"5V series current-limiting resistor for blue LED D2.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2},{"reference":"R24","purpose_zh":"D3 藍光 LED 的 5V 串聯限流電阻。","purpose_en":"5V series current-limiting resistor for blue LED D3.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2},{"reference":"R29","purpose_zh":"U8 輸出至 ADC_AINP 的串聯隔離／濾波电阻。","purpose_en":"Series isolation/filtering resistor from U8 output to ADC_AINP.","location_zh":"原理圖第 2 頁：TIA／ADC","location_en":"Schematic page 2: TIA / ADC","page":2},{"reference":"R30","purpose_zh":"D4 藍光 LED 的 5V 串聯限流電阻。","purpose_en":"5V series current-limiting resistor for blue LED D4.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2},{"reference":"R31","purpose_zh":"3V3_ANA 至 U8 局部供電的串聯濾波電阻，搭配 C25/C26。","purpose_en":"Series supply-filter resistor from 3V3_ANA to the U8 local supply, used with C25/C26.","location_zh":"原理圖第 2 頁：TIA</x:v>
+      </x:c>
+      <x:c r="C159" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="264" customHeight="1">
+      <x:c r="A160" s="18" t="str">
+        <x:v>45: R16,R21,R24,R29,R30,R31,R3
+6 （續）</x:v>
+      </x:c>
+      <x:c r="B160" s="18" t="str">
+        <x:v> 供電","location_en":"Schematic page 2: TIA supply","page":2},{"reference":"R36","purpose_zh":"ADC_AINN 至 GND 的串聯電阻，搭配 R29/C24 的輸入網路。","purpose_en":"Series resistor from ADC_AINN to ground in the R29/C24 input network.","location_zh":"原理圖第 2 頁：TIA／ADC","location_en":"Schematic page 2: TIA / ADC","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱阻值 100R。","spec_en":"Vendor nominal resistance: 100R.","purpose_zh":"R16: D1 藍光 LED 的 5V 串聯限流電阻。；R21: D2 藍光 LED 的 5V 串聯限流電阻。；R24: D3 藍光 LED 的 5V 串聯限流電阻。；R29: U8 輸出至 ADC_AINP 的串聯隔離／濾波电阻。；R30: D4 藍光 LED 的 5V 串聯限流電阻。；R31: 3V3_ANA 至 U8 局部供電的串聯濾波電阻，搭配 C25/C26。；R36: ADC_AINN 至 GND 的串聯電阻，搭配 R29/C24 的輸入網路。","purpose_en":"R16: 5V series current-limiting resistor for blue LED D1.；R21: 5V series current-limiting resistor for blue LED D2.；R24: 5V series current-limiting resistor for blue LED D3.；R29: Series isolation/filtering resistor from U8 output to ADC_AINP.；R30: 5V series current-limiting resistor for blue LED D4.；R31: Series supply-filter resistor from 3V3_ANA to the U8 local supply, used with C25/C26.；R36: Series resistor from ADC_AINN to ground in the R29/C24 input network.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 45</x:v>
+      </x:c>
+      <x:c r="C160" s="18" t="str"/>
+    </x:row>
+    <x:row r="161" ht="180" customHeight="1">
+      <x:c r="A161" s="18" t="str">
+        <x:v>46: R17,R22,R25,R32</x:v>
+      </x:c>
+      <x:c r="B161" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 46
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R17","purpose_zh":"LED1_GATE 至 Q1 閘極的串聯電阻。","purpose_en":"Series resistor from LED1_GATE to the Q1 gate.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2},{"reference":"R22","purpose_zh":"LED2_GATE 至 Q2 閘極的串聯電阻。","purpose_en":"Series resistor from LED2_GATE to the Q2 gate.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2},{"reference":"R25","purpose_zh":"LED3_GATE 至 Q3 閘極的串聯電阻。","purpose_en":"Series resistor from LED3_GATE to the Q3 gate.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2},{"reference":"R32","purpose_zh":"LED4_GATE 至 Q4 閘極的串聯電阻。","purpose_en":"Series resistor from LED4_GATE to</x:v>
+      </x:c>
+      <x:c r="C161" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="166" customHeight="1">
+      <x:c r="A162" s="18" t="str">
+        <x:v>46: R17,R22,R25,R32 （續）</x:v>
+      </x:c>
+      <x:c r="B162" s="18" t="str">
+        <x:v> the Q4 gate.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱阻值 220R。","spec_en":"Vendor nominal resistance: 220R.","purpose_zh":"R17: LED1_GATE 至 Q1 閘極的串聯電阻。；R22: LED2_GATE 至 Q2 閘極的串聯電阻。；R25: LED3_GATE 至 Q3 閘極的串聯電阻。；R32: LED4_GATE 至 Q4 閘極的串聯電阻。","purpose_en":"R17: Series resistor from LED1_GATE to the Q1 gate.；R22: Series resistor from LED2_GATE to the Q2 gate.；R25: Series resistor from LED3_GATE to the Q3 gate.；R32: Series resistor from LED4_GATE to the Q4 gate.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 46</x:v>
+      </x:c>
+      <x:c r="C162" s="18" t="str"/>
+    </x:row>
+    <x:row r="163" ht="180" customHeight="1">
+      <x:c r="A163" s="18" t="str">
+        <x:v>47: R20,R23,R26,R33</x:v>
+      </x:c>
+      <x:c r="B163" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 47
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R20","purpose_zh":"Q1 閘極至源極／GND 的下拉。","purpose_en":"Pull-down from the Q1 gate to its source / ground.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2},{"reference":"R23","purpose_zh":"Q2 閘極至源極／GND 的下拉。","purpose_en":"Pull-down from the Q2 gate to its source / ground.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2},{"reference":"R26","purpose_zh":"Q3 閘極至源極／GND 的下拉。","purpose_en":"Pull-down from the Q3 gate to its source / ground.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2},{"reference":"R33","purpose_zh":"Q4 閘極至源極／GND 的下拉。","purpose_en":"Pull-down from the Q4 gate to its</x:v>
+      </x:c>
+      <x:c r="C163" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="180" customHeight="1">
+      <x:c r="A164" s="18" t="str">
+        <x:v>47: R20,R23,R26,R33 （續）</x:v>
+      </x:c>
+      <x:c r="B164" s="18" t="str">
+        <x:v> source / ground.","location_zh":"原理圖第 2 頁：LEDs","location_en":"Schematic page 2: LEDs","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱阻值 100k。","spec_en":"Vendor nominal resistance: 100k.","purpose_zh":"R20: Q1 閘極至源極／GND 的下拉。；R23: Q2 閘極至源極／GND 的下拉。；R26: Q3 閘極至源極／GND 的下拉。；R33: Q4 閘極至源極／GND 的下拉。","purpose_en":"R20: Pull-down from the Q1 gate to its source / ground.；R23: Pull-down from the Q2 gate to its source / ground.；R26: Pull-down from the Q3 gate to its source / ground.；R33: Pull-down from the Q4 gate to its source / ground.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 47</x:v>
+      </x:c>
+      <x:c r="C164" s="18" t="str"/>
+    </x:row>
+    <x:row r="165" ht="264" customHeight="1">
+      <x:c r="A165" s="18" t="str">
+        <x:v>48: R27</x:v>
+      </x:c>
+      <x:c r="B165" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 30
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 48
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R27","purpose_zh":"U8 輸出至反相輸入的跨阻回授電阻，將 PD 光電流轉成電壓；與 C21 並聯。","purpose_en":"Transimpedance feedback from U8 output to its inverting input, converting PD photocurrent to voltage; in parallel with C21.","location_zh":"原理圖第 2 頁：TIA","location_en":"Schematic page 2: TIA","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱阻值 100M。","spec_en":"Vendor nominal resistance: 100M.","purpose_zh":"R27: U8 輸出至反相輸入的跨阻回授電阻，將 PD 光電流轉成電壓；與 C21 並聯。","purpose_en":"R27: Transimpedance feedback from U8 output to its inverting input, converting PD photocurrent to voltage; in parallel with C21.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。 100 MΩ 回授需另核對漏電、清潔／濕度敏感度與雜訊；不可僅凭阻值任選。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied. The 100 MΩ feedback also requires leakage, cleaning/humidity and noise review; resistance alone is insufficient."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 48</x:v>
+      </x:c>
+      <x:c r="C165" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="236" customHeight="1">
+      <x:c r="A166" s="18" t="str">
+        <x:v>49: R34</x:v>
+      </x:c>
+      <x:c r="B166" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 5
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 49
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R34","purpose_zh":"與 C28 串聯接於 VREF_2V5 至 GND 旁路支路；不是電流感測電阻，也非串在 ADC 訊號線中。","purpose_en":"In series with C28 in the VREF_2V5-to-ground bypass branch; not a current-sense resistor or series ADC-signal resistor.","location_zh":"原理圖第 2 頁：ADC 參考","location_en":"Schematic page 2: ADC reference","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱阻值 0.1R。","spec_en":"Vendor nominal resistance: 0.1R.","purpose_zh":"R34: 與 C28 串聯接於 VREF_2V5 至 GND 旁路支路；不是電流感測電阻，也非串在 ADC 訊號線中。","purpose_en":"R34: In series with C28 in the VREF_2V5-to-ground bypass branch; not a current-sense resistor or series ADC-signal resistor.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 49</x:v>
+      </x:c>
+      <x:c r="C166" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="264" customHeight="1">
+      <x:c r="A167" s="18" t="str">
+        <x:v>50: R37,R38</x:v>
+      </x:c>
+      <x:c r="B167" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 1
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 50
+source_ids: ["vendor_BOM","schematic"]
+per_reference: [{"reference":"R37","purpose_zh":"ESP32 ADC_SCLK 至 U9 SCLK 的串聯電阻。","purpose_en":"Series resistor from ESP32 ADC_SCLK to U9 SCLK.","location_zh":"原理圖第 2 頁：ADC 數位介面","location_en":"Schematic page 2: ADC digital interface","page":2},{"reference":"R38","purpose_zh":"ESP32 ADC_CONVST 至 U9 CONVST 的串聯電阻。","purpose_en":"Series resistor from ESP32 ADC_CONVST to U9 CONVST.","location_zh":"原理圖第 2 頁：ADC 數位介面","location_en":"Schematic page 2: ADC digital interface","page":2}]
+orderability: incomplete_passive_specification
+details: {"spec_zh":"原廠標稱阻值 47R。","spec_en":"Vendor nominal resistance: 47R.","purpose_zh":"R37: ESP32 ADC_SCLK 至 U9 SCLK 的串聯電阻。；R38: ESP32 ADC_CONVST 至 U9 CONVST 的串聯電阻。","purpose_en":"R37: Series resistor from ESP32 ADC_SCLK to U9 SCLK.；R38: Series resistor from ESP32 ADC_CONVST to U9 CONVST.","missing_zh":"廠牌／完整料號、封裝尺寸與高度、功率、容差、溫度係數及最大工作電壓尚未提供。","missing_en":"Manufacturer/orderable MPN, case dimensions/height, power rating, tolerance, temperature coefficient and maximum working voltage are not supplied."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 50</x:v>
+      </x:c>
+      <x:c r="C167" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="208" customHeight="1">
+      <x:c r="A168" s="18" t="str">
+        <x:v>51: SW1</x:v>
+      </x:c>
+      <x:c r="B168" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 15
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 51
+source_ids: ["vendor_BOM","schematic"]
+per_reference: []
+orderability: incomplete_component_specification
+details: {"spec_zh":"原圖三接點 COMM/B/A；COMM 接系統供電，B 經 R4 接 EN，A 未接。","spec_en":"Three schematic contacts COMM/B/A; COMM is at system supply, B connects through R4 to EN, and A is unconnected.","purpose_zh":"切換 U1 升壓啟用控制；不能據此宣稱切斷 USB 充電器或所有電池電流。","purpose_en":"Switches the U1 boost-enable control; it does not establish isolation of the USB charger or all battery current.","missing_zh":"MPN、實體型式、封裝／操作柄位置與行程、額定值及開孔尺寸未提供。","missing_en":"MPN, physical type, footprint/actuator position and travel, ratings and panel opening are unspecified."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 51</x:v>
+      </x:c>
+      <x:c r="C168" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="180" customHeight="1">
+      <x:c r="A169" s="18" t="str">
+        <x:v>52: SW2,SW3</x:v>
+      </x:c>
+      <x:c r="B169" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+unit_price: 5
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 52
+source_ids: ["vendor_BOM","schematic"]
+per_reference: []
+orderability: incomplete_component_specification
+details: {"spec_zh":"SW2、SW3；原圖按下時將各訊號接 GND。","spec_en":"SW2 and SW3; each grounds its respective signal when pressed.","purpose_zh":"SW2：ESP_EN 復位；SW3：ESP_IO0 啟動／下載模式選擇。","purpose_en":"SW2: ESP_EN reset; SW3: ESP_IO0 boot/download-mode selection.","missing_zh":"完整MPN、接點規格、封裝尺寸／按壓高度／方向、操作力與壽命未提供。","missing_en":"MPN, contact rating, footprint/actuation height/direction, force and life are unspecified."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 52</x:v>
+      </x:c>
+      <x:c r="C169" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="208" customHeight="1">
+      <x:c r="A170" s="18" t="str">
+        <x:v>53: U1</x:v>
+      </x:c>
+      <x:c r="B170" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 52
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 53
+source_ids: ["vendor_BOM","schematic","TI_TPS61023"]
+per_reference: []
+orderability: identified_part_pending_assembly_verification
+details: {"spec_zh":"TI TPS61023；6-pin SOT-563 (DRL)。3.7 A 指開關電流限制，不能當作5 V輸出額定電流。","spec_en":"TI TPS61023; 6-pin SOT-563 (DRL). The 3.7 A figure is a switch-current limit, not a 5 V output-current rating.","purpose_zh":"將充電器 OUT／電池系統供電升壓至圖示5V軌，供 LED 與後級 LDO。","purpose_en":"Boosts the charger OUT / battery-system supply to the rail labelled 5V for LEDs and downstream LDOs.","missing_zh":"完整訂購後綴、L1/C2–C5/R6/R8 等值未完整提供；5V設定、穩定度及風扇可用電流須廠商驗證。","missing_en":"Full ordering suffix and L1/C2–C5/R6/R8 values are incomplete; vendor must validate the 5V setting, stability and available fan current."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 53</x:v>
+      </x:c>
+      <x:c r="C170" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="208" customHeight="1">
+      <x:c r="A171" s="18" t="str">
+        <x:v>54: U2</x:v>
+      </x:c>
+      <x:c r="B171" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 88
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 54
+source_ids: ["vendor_BOM","schematic","TI_BQ24074"]
+per_reference: []
+orderability: identified_part_pending_assembly_verification
+details: {"spec_zh":"TI BQ24074；4.2 V 單節 Li-ion/Li-poly 充電器；16-pin VQFN (RGT)，3×3 mm。","spec_en":"TI BQ24074; 4.2 V single-cell Li-ion/Li-poly charger; 16-pin VQFN (RGT), 3×3 mm.","purpose_zh":"接 USB 5V_USB、BAT 電池與 OUT 系統供電；OUT 不是已調節的5 V升壓輸出。","purpose_en":"Interfaces USB 5V_USB, the BAT battery node and OUT system supply; OUT is not the regulated 5V boost output.","missing_zh":"完整訂購後綴、R1/R2/R3/R9 及電池／散熱配置未定；不可將器件1.5 A能力當作本板已設定充電電流。","missing_en":"Full ordering suffix, R1/R2/R3/R9, cell and thermal configuration remain incomplete; the device 1.5 A capability is not the configured board charging current."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 54</x:v>
+      </x:c>
+      <x:c r="C171" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="194" customHeight="1">
+      <x:c r="A172" s="18" t="str">
+        <x:v>55: U3</x:v>
+      </x:c>
+      <x:c r="B172" s="18" t="str">
+        <x:v>status: 規格/MPN未完整
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 55
+source_ids: ["vendor_BOM","schematic"]
+per_reference: []
+orderability: unidentified_component
+details: {"spec_zh":"原廠僅有 U3、P1–P6；無型號或功能名稱。","spec_en":"Only U3 and P1–P6 are provided; no MPN or functional identity.","purpose_zh":"P1 接系統供電、P5 接 GND、P2 接 R10/R12/C9、P3 接升壓 EN，P4/P6 各接電容至GND。功能必須由廠商確認。","purpose_en":"P1 connects to system supply, P5 to ground, P2 to R10/R12/C9, P3 to boost EN, and P4/P6 each to a capacitor to ground. Vendor identification is required.","missing_zh":"IC 類型、完整MPN、供電／輸出額定值、腳位定義、封裝與周邊值皆未定；不能指定替代料。","missing_en":"IC type, MPN, supply/output ratings, pin functions, package and external values are unknown; no substitute can be specified."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 55</x:v>
+      </x:c>
+      <x:c r="C172" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="222" customHeight="1">
+      <x:c r="A173" s="18" t="str">
+        <x:v>56: U4</x:v>
+      </x:c>
+      <x:c r="B173" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 181
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 56
+source_ids: ["vendor_BOM","schematic","ESPRESSIF_32E"]
+per_reference: []
+orderability: identified_part_pending_assembly_verification
+details: {"spec_zh":"Espressif ESP32-WROOM-32E；2.4 GHz 無線、3.3 V 系統模組；32E 為板載 PCB 天線版本。","spec_en":"Espressif ESP32-WROOM-32E; 2.4 GHz wireless module for a 3.3 V system; 32E uses an onboard PCB antenna.","purpose_zh":"控制四路 LED、讀取 ADS8866 並提供網路介面；原圖 UART 在 J3。","purpose_en":"Controls four LED channels, reads ADS8866 and provides networking; schematic UART is available at J3.","missing_zh":"需確認完整容量／溫度等訂購後綴、實際焊接高度與天線禁布／外殼空間；不要把32E誤當具外接天線座的32UE。","missing_en":"Confirm the full flash/temperature ordering variant, assembled height and antenna keepout/enclosure clearance; do not confuse 32E with the external-antenna-connector 32UE."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 56</x:v>
+      </x:c>
+      <x:c r="C173" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="208" customHeight="1">
+      <x:c r="A174" s="18" t="str">
+        <x:v>57: U5</x:v>
+      </x:c>
+      <x:c r="B174" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 10
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 57
+source_ids: ["vendor_BOM","schematic","ECMOS_EC50117"]
+per_reference: []
+orderability: identified_part_pending_assembly_verification
+details: {"spec_zh":"E-CMOS EC50117KBG；官方訂購表確認固定3.3 V、SOT-223；系列標稱1 A能力。","spec_en":"E-CMOS EC50117KBG; manufacturer ordering table identifies fixed 3.3 V, SOT-223; series nominal 1 A capability.","purpose_zh":"5V 輸入轉為 3V3_DIG，供 ESP32 與數位電路。","purpose_en":"Converts the 5V input to 3V3_DIG for ESP32 and digital circuitry.","missing_zh":"實際可用電流取決於壓差、PCB散熱與負載；須核對 C17/C18 型式、穩定性與組裝封裝，不能宣稱本板可持續供1 A。","missing_en":"Available current depends on dropout, PCB cooling and load; verify C17/C18 type, stability and assembled package. Continuous 1 A board output is not established."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 57</x:v>
+      </x:c>
+      <x:c r="C174" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="208" customHeight="1">
+      <x:c r="A175" s="18" t="str">
+        <x:v>58: U6</x:v>
+      </x:c>
+      <x:c r="B175" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 24
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 58
+source_ids: ["vendor_BOM","schematic","TI_LP5907"]
+per_reference: []
+orderability: identified_part_pending_assembly_verification
+details: {"spec_zh":"TI LP5907MFX-3.3/NOPB；固定3.3 V、250 mA 器件額定能力；5-pin SOT-23 (DBV)。","spec_en":"TI LP5907MFX-3.3/NOPB; fixed 3.3 V, 250 mA device capability; 5-pin SOT-23 (DBV).","purpose_zh":"將5V轉為3V3_ANA，供類比前端、ADC類比電源及參考電壓IC；EN 接輸入。","purpose_en":"Generates 3V3_ANA from 5V for the analog front end, ADC analog supply and reference IC; EN is tied to input.","missing_zh":"須核對C19/C20有效容值、穩定性、熱耗散與封裝焊盘；額定250 mA不是全系統驗證結果。","missing_en":"Verify effective C19/C20 capacitance, stability, dissipation and footprint; the 250 mA rating is not a whole-system validation result."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 58</x:v>
+      </x:c>
+      <x:c r="C175" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" ht="208" customHeight="1">
+      <x:c r="A176" s="18" t="str">
+        <x:v>59: U7</x:v>
+      </x:c>
+      <x:c r="B176" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 628
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 59
+source_ids: ["vendor_BOM","schematic","ADI_LTC6655"]
+per_reference: []
+orderability: identified_part_pending_assembly_verification
+details: {"spec_zh":"Analog Devices LTC6655BHMS8-2.5#PBF；2.5 V 輸出、8-pin MSOP。","spec_en":"Analog Devices LTC6655BHMS8-2.5#PBF; 2.5 V output, 8-pin MSOP.","purpose_zh":"由3V3_ANA產生VREF_2V5，供U9 ADC参考；SHDN經R28上拉，輸出force/sense腳於圖中相接。","purpose_en":"Generates VREF_2V5 from 3V3_ANA for U9; SHDN is pulled up by R28 and output force/sense pins are joined in the schematic.","missing_zh":"須核對C22/C23型式、負載／穩定性、佈線與ADC實際參考電壓；不可把名義2.5 V當作已校準量測。","missing_en":"Verify C22/C23 type, load/stability, layout and measured ADC reference voltage; nominal 2.5 V is not a calibrated measurement."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 59</x:v>
+      </x:c>
+      <x:c r="C176" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="208" customHeight="1">
+      <x:c r="A177" s="18" t="str">
+        <x:v>60: U8</x:v>
+      </x:c>
+      <x:c r="B177" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 226
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 60
+source_ids: ["vendor_BOM","schematic","TI_LMP7721"]
+per_reference: []
+orderability: identified_part_pending_assembly_verification
+details: {"spec_zh":"TI LMP7721；單運算放大器、8-pin SOIC (D)，供電範圍1.8–5.5 V。","spec_en":"TI LMP7721; single amplifier, 8-pin SOIC (D), 1.8–5.5 V supply range.","purpose_zh":"U8以R27=100 MΩ／C21=2.2 pF跨阻回授讀取D5；非反相端接GND，供電經R31/C25/C26濾波。","purpose_en":"U8 reads D5 using R27=100 MΩ / C21=2.2 pF transimpedance feedback; its non-inverting input is grounded and supply is filtered by R31/C25/C26.","missing_zh":"完整訂購後綴、實際封裝與低漏電佈線／清潔、穩定性和接近地電位輸出範圍需驗證；此表不等於TIA性能驗證。","missing_en":"Confirm full ordering suffix, package, low-leakage layout/cleanliness, stability and near-ground output range; this BOM is not TIA performance validation."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 60</x:v>
+      </x:c>
+      <x:c r="C177" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="208" customHeight="1">
+      <x:c r="A178" s="18" t="str">
+        <x:v>61: U9</x:v>
+      </x:c>
+      <x:c r="B178" s="18" t="str">
+        <x:v>status: 依廠商BOM，封裝/容差仍需確認
+unit_price: 306
+source: NTHU_TEST_BOARD_BOM.docx vendor table row 61
+source_ids: ["vendor_BOM","schematic","TI_ADS8866"]
+per_reference: []
+orderability: identified_part_pending_assembly_verification
+details: {"spec_zh":"TI ADS8866IDGS；16-bit、100 kSPS 器件上限，10-pin VSSOP (DGS)；外接參考。","spec_en":"TI ADS8866IDGS; 16-bit, 100 kSPS device limit, 10-pin VSSOP (DGS); external reference.","purpose_zh":"取樣TIA輸出；AVDD=3V3_ANA、DVDD=3V3_DIG、REF=VREF_2V5；SCLK/DOUT/CONVST接ESP32。","purpose_en":"Samples TIA output; AVDD=3V3_ANA, DVDD=3V3_DIG, REF=VREF_2V5; SCLK/DOUT/CONVST interface to ESP32.","missing_zh":"需確認實際取樣率／時序、ADC輸入建立時間與雜訊、參考與電源去耦；100 kSPS不是目前韌體已驗證的取樣性能。","missing_en":"Verify actual sampling/timing, input settling/noise and reference/supply decoupling; 100 kSPS is not verified current firmware performance."}
+original_source: NTHU_TEST_BOARD_BOM.docx vendor table row 61</x:v>
+      </x:c>
+      <x:c r="C178" s="18" t="str">
+        <x:v>原供應商／來源欄位；採用 PCB 工作表的現行估值與待確認規格。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="30" customHeight="1">
+      <x:c r="A179" s="25" t="str">
+        <x:v>列印幾何與檔案識別</x:v>
+      </x:c>
+      <x:c r="B179" s="25" t="str"/>
+      <x:c r="C179" s="25" t="str"/>
+    </x:row>
+    <x:row r="180" ht="110" customHeight="1">
+      <x:c r="A180" s="18" t="str">
+        <x:v>01_base_BLACK.stl</x:v>
+      </x:c>
+      <x:c r="B180" s="18" t="str">
+        <x:v>Batch: P1
+Triangles: 7248; connected components: 1; watertight edges: true
+Mesh volume: 78.13914674155713 cm3
+Assembly minimum: -54, -56, 0 mm
+Assembly maximum: 54, 52, 43.29999923706055 mm
+Size: 108, 108, 43.29999923706055 mm
+Degenerate triangles removed in original export: 0</x:v>
+      </x:c>
+      <x:c r="C180" s="18" t="str">
+        <x:v>SHA256: dd90fa4a126e02d6523114ea447e4f24aaf27826d7a456a111bd6cf6feee2b22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="110" customHeight="1">
+      <x:c r="A181" s="18" t="str">
+        <x:v>02_black_hood_BLACK.stl</x:v>
+      </x:c>
+      <x:c r="B181" s="18" t="str">
+        <x:v>Batch: P2
+Triangles: 1976; connected components: 1; watertight edges: true
+Mesh volume: 28.76661897830055 cm3
+Assembly minimum: -54, -56, 40.79999923706055 mm
+Assembly maximum: 54, 52, 64 mm
+Size: 108, 108, 23.200000762939453 mm
+Degenerate triangles removed in original export: 0</x:v>
+      </x:c>
+      <x:c r="C181" s="18" t="str">
+        <x:v>SHA256: c45b0cded88cfa45070e5f04c933d58ffb0aead62d7ea7d8899ca5c906f7f557</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="110" customHeight="1">
+      <x:c r="A182" s="18" t="str">
+        <x:v>03_gas_lid_BLACK.stl</x:v>
+      </x:c>
+      <x:c r="B182" s="18" t="str">
+        <x:v>Batch: P2
+Triangles: 3372; connected components: 1; watertight edges: true
+Mesh volume: 29.53238239220095 cm3
+Assembly minimum: -54, -56, 57.900001525878906 mm
+Assembly maximum: 54, 52, 66 mm
+Size: 108, 108, 8.099998474121094 mm
+Degenerate triangles removed in original export: 2</x:v>
+      </x:c>
+      <x:c r="C182" s="18" t="str">
+        <x:v>SHA256: eb1af20eb3458d72ddc2b2a70a6b206e97616f6d677a2dc703a870ec99c691dd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="110" customHeight="1">
+      <x:c r="A183" s="18" t="str">
+        <x:v>04_well_NE_CLEAR.stl</x:v>
+      </x:c>
+      <x:c r="B183" s="18" t="str">
+        <x:v>Batch: P3
+Triangles: 40; connected components: 1; watertight edges: true
+Mesh volume: 0.11564499290465757 cm3
+Assembly minimum: 0.7999992370605469, 0.75, 42.5 mm
+Assembly maximum: 6.5, 5.25, 55.5 mm
+Size: 5.700000762939453, 4.5, 13 mm
+Degenerate triangles removed in original export: 0</x:v>
+      </x:c>
+      <x:c r="C183" s="18" t="str">
+        <x:v>SHA256: b349bc6ee902d8bdb5c7e42d39c7ebe928e01e4c2a883a2d869645bee29c86c7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="110" customHeight="1">
+      <x:c r="A184" s="18" t="str">
+        <x:v>05_well_NW_CLEAR.stl</x:v>
+      </x:c>
+      <x:c r="B184" s="18" t="str">
+        <x:v>Batch: P3
+Triangles: 40; connected components: 1; watertight edges: true
+Mesh volume: 0.1156449929046576 cm3
+Assembly minimum: -6.5, 0.75, 42.5 mm
+Assembly maximum: -0.7999992370605469, 5.25, 55.5 mm
+Size: 5.700000762939453, 4.5, 13 mm
+Degenerate triangles removed in original export: 0</x:v>
+      </x:c>
+      <x:c r="C184" s="18" t="str">
+        <x:v>SHA256: c4d0085d0fd145611bef334bfc3ec3b513f1340f9608a29822ac0ccd709bb790</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="110" customHeight="1">
+      <x:c r="A185" s="18" t="str">
+        <x:v>06_well_SW_CLEAR.stl</x:v>
+      </x:c>
+      <x:c r="B185" s="18" t="str">
+        <x:v>Batch: P3
+Triangles: 40; connected components: 1; watertight edges: true
+Mesh volume: 0.11564499290465756 cm3
+Assembly minimum: -6.5, -5.25, 42.5 mm
+Assembly maximum: -0.7999992370605469, -0.75, 55.5 mm
+Size: 5.700000762939453, 4.5, 13 mm
+Degenerate triangles removed in original export: 0</x:v>
+      </x:c>
+      <x:c r="C185" s="18" t="str">
+        <x:v>SHA256: fec68336b7a5b404f66f46e0a54f6d66ed84ff590e85e4793ce028ff90a10fb2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="110" customHeight="1">
+      <x:c r="A186" s="18" t="str">
+        <x:v>07_well_SE_CLEAR.stl</x:v>
+      </x:c>
+      <x:c r="B186" s="18" t="str">
+        <x:v>Batch: P3
+Triangles: 40; connected components: 1; watertight edges: true
+Mesh volume: 0.11564499290465757 cm3
+Assembly minimum: 0.7999992370605469, -5.25, 42.5 mm
+Assembly maximum: 6.5, -0.75, 55.5 mm
+Size: 5.700000762939453, 4.5, 13 mm
+Degenerate triangles removed in original export: 0</x:v>
+      </x:c>
+      <x:c r="C186" s="18" t="str">
+        <x:v>SHA256: 64930ddaca73a7cfd28599e3525a9e77f26db9e8bbb255e126343b579945a363</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="110" customHeight="1">
+      <x:c r="A187" s="18" t="str">
+        <x:v>08_gas_compression_plate_B
+LACK.stl</x:v>
+      </x:c>
+      <x:c r="B187" s="18" t="str">
+        <x:v>Batch: P2
+Triangles: 92; connected components: 1; watertight edges: true
+Mesh volume: 0.37824025512696247 cm3
+Assembly minimum: -10, -9, 56.099998474121094 mm
+Assembly maximum: 10, 9, 57.29999923706055 mm
+Size: 20, 18, 1.2000007629394531 mm
+Degenerate triangles removed in original export: 0</x:v>
+      </x:c>
+      <x:c r="C187" s="18" t="str">
+        <x:v>SHA256: 8255ef667a516ba1fd46389974d341523e5bcee4bc5f81e6805fa2f3b864ef64</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="28" customHeight="1">
+      <x:c r="A188" s="18" t="str">
+        <x:v>01_base_BLACK.ctb</x:v>
+      </x:c>
+      <x:c r="B188" s="18" t="str">
+        <x:v>切片列印檔。整理前後位元組內容相同。</x:v>
+      </x:c>
+      <x:c r="C188" s="18" t="str">
+        <x:v>SHA256: 1d05971e924c78ade7c83b0acae26120e2dddff5b3b52b35064b252af4ad474b</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="28" customHeight="1">
+      <x:c r="A189" s="18" t="str">
+        <x:v>020308_parts.ctb</x:v>
+      </x:c>
+      <x:c r="B189" s="18" t="str">
+        <x:v>切片列印檔。整理前後位元組內容相同。</x:v>
+      </x:c>
+      <x:c r="C189" s="18" t="str">
+        <x:v>SHA256: f76017570fd0f2680b0245193d79bfe6ccc4f6919abb938166f5a0cc9a814a6e</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" ht="28" customHeight="1">
+      <x:c r="A190" s="18" t="str">
+        <x:v>0407_wells.ctb</x:v>
+      </x:c>
+      <x:c r="B190" s="18" t="str">
+        <x:v>切片列印檔。整理前後位元組內容相同。</x:v>
+      </x:c>
+      <x:c r="C190" s="18" t="str">
+        <x:v>SHA256: cec360f96ba4704f76ac404b8af52bdb09c2033c37464cb0cb0512ec80cab98d</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="30" customHeight="1">
+      <x:c r="A191" s="25" t="str">
+        <x:v>計價原則</x:v>
+      </x:c>
+      <x:c r="B191" s="25" t="str"/>
+      <x:c r="C191" s="25" t="str"/>
+    </x:row>
+    <x:row r="192" ht="28" customHeight="1">
+      <x:c r="A192" s="18" t="str">
+        <x:v>quantity_basis</x:v>
+      </x:c>
+      <x:c r="B192" s="18" t="str">
+        <x:v>Small-quantity retail; listings, proxies and allowances explicitly distinguished</x:v>
+      </x:c>
+      <x:c r="C192" s="18" t="str"/>
+    </x:row>
+    <x:row r="193" ht="28" customHeight="1">
+      <x:c r="A193" s="18" t="str">
+        <x:v>tax_shipping</x:v>
+      </x:c>
+      <x:c r="B193" s="18" t="str">
+        <x:v>Shipping, import duties and taxes not included unless source explicitly states included</x:v>
+      </x:c>
+      <x:c r="C193" s="18" t="str"/>
+    </x:row>
+    <x:row r="194" ht="28" customHeight="1">
+      <x:c r="A194" s="18" t="str">
+        <x:v>PCBA</x:v>
+      </x:c>
+      <x:c r="B194" s="18" t="str">
+        <x:v>Use quoted allocation once; do not add PCB component estimate again</x:v>
+      </x:c>
+      <x:c r="C194" s="18" t="str"/>
+    </x:row>
+    <x:row r="195" ht="28" customHeight="1">
+      <x:c r="A195" s="18" t="str">
+        <x:v>printing</x:v>
+      </x:c>
+      <x:c r="B195" s="18" t="str">
+        <x:v>Preserve user formula and source amounts; no extra bottle cost or machine charge added</x:v>
+      </x:c>
+      <x:c r="C195" s="18" t="str"/>
+    </x:row>
+    <x:row r="196" ht="28" customHeight="1">
+      <x:c r="A196" s="18" t="str">
+        <x:v>future</x:v>
+      </x:c>
+      <x:c r="B196" s="18" t="str">
+        <x:v>Excluded from current device and development totals</x:v>
+      </x:c>
+      <x:c r="C196" s="18" t="str"/>
+    </x:row>
+    <x:row r="197" ht="28" customHeight="1">
+      <x:c r="A197" s="18" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="B197" s="18" t="str">
+        <x:v>Unidentified U3 not assigned a false price; custom optical filter not order-ready</x:v>
+      </x:c>
+      <x:c r="C197" s="18" t="str"/>
+    </x:row>
+    <x:row r="198" ht="28" customHeight="1">
+      <x:c r="A198" s="18" t="str">
+        <x:v>owned</x:v>
+      </x:c>
+      <x:c r="B198" s="18" t="str">
+        <x:v>owned_qty editable. Borrowed items can reduce new purchase budget without making material value zero.</x:v>
+      </x:c>
+      <x:c r="C198" s="18" t="str"/>
+    </x:row>
+    <x:row r="199" ht="28" customHeight="1">
+      <x:c r="A199" s="18" t="str">
+        <x:v>PCB 報價範圍</x:v>
+      </x:c>
+      <x:c r="B199" s="18" t="str">
+        <x:v>User quotation including design and setup; per-board allocation is not repeat-production pricing</x:v>
+      </x:c>
+      <x:c r="C199" s="18" t="str">
+        <x:v>原報價 NTD 131250／2 片。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200" ht="40" customHeight="1">
+      <x:c r="A200" s="18" t="str">
+        <x:v>匯率來源紀錄</x:v>
+      </x:c>
+      <x:c r="B200" s="18" t="str">
+        <x:v>31.805 NTD per USD; source date 2026-10-05 15:13; recorded 2026-10-08.
+Bank of Taiwan displayed USD spot selling snapshot; comparison and budgeting only</x:v>
+      </x:c>
+      <x:c r="C200" s="18" t="str">
+        <x:v>https://www.bot.com.tw/tw/personal-banking/foreign-exchange</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201" ht="30" customHeight="1">
+      <x:c r="A201" s="25" t="str">
+        <x:v>歷史驗證紀錄</x:v>
+      </x:c>
+      <x:c r="B201" s="25" t="str"/>
+      <x:c r="C201" s="25" t="str"/>
+    </x:row>
+    <x:row r="202" ht="28" customHeight="1">
+      <x:c r="A202" s="18" t="str">
+        <x:v>範圍</x:v>
+      </x:c>
+      <x:c r="B202" s="18" t="str">
+        <x:v>下列欄位描述此次整併前的既有工作簿。舊雜湊只識別先前版本，不代表已在原生 Excel 執行。</x:v>
+      </x:c>
+      <x:c r="C202" s="18" t="str"/>
+    </x:row>
+    <x:row r="203" ht="28" customHeight="1">
+      <x:c r="A203" s="18" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="B203" s="18" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="C203" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="28" customHeight="1">
+      <x:c r="A204" s="18" t="str">
+        <x:v>formula_engine</x:v>
+      </x:c>
+      <x:c r="B204" s="18" t="str">
+        <x:v>artifact-tool</x:v>
+      </x:c>
+      <x:c r="C204" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205" ht="40" customHeight="1">
+      <x:c r="A205" s="18" t="str">
+        <x:v>native_Excel_execution_ver
+ified</x:v>
+      </x:c>
+      <x:c r="B205" s="18" t="str">
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="C205" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206" ht="28" customHeight="1">
+      <x:c r="A206" s="18" t="str">
+        <x:v>print_count</x:v>
+      </x:c>
+      <x:c r="B206" s="18" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C206" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207" ht="28" customHeight="1">
+      <x:c r="A207" s="18" t="str">
+        <x:v>PCB_rows</x:v>
+      </x:c>
+      <x:c r="B207" s="18" t="str">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="C207" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208" ht="28" customHeight="1">
+      <x:c r="A208" s="18" t="str">
+        <x:v>purchase_rows</x:v>
+      </x:c>
+      <x:c r="B208" s="18" t="str">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="C208" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" ht="28" customHeight="1">
+      <x:c r="A209" s="18" t="str">
+        <x:v>required_rows</x:v>
+      </x:c>
+      <x:c r="B209" s="18" t="str">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C209" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210" ht="28" customHeight="1">
+      <x:c r="A210" s="18" t="str">
+        <x:v>developer_rows</x:v>
+      </x:c>
+      <x:c r="B210" s="18" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C210" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211" ht="28" customHeight="1">
+      <x:c r="A211" s="18" t="str">
+        <x:v>future_rows</x:v>
+      </x:c>
+      <x:c r="B211" s="18" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C211" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="28" customHeight="1">
+      <x:c r="A212" s="18" t="str">
+        <x:v>calculated_print_total_TWD</x:v>
+      </x:c>
+      <x:c r="B212" s="18" t="str">
+        <x:v>1115.3856</x:v>
+      </x:c>
+      <x:c r="C212" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="28" customHeight="1">
+      <x:c r="A213" s="18" t="str">
+        <x:v>known_required_low_TWD</x:v>
+      </x:c>
+      <x:c r="B213" s="18" t="str">
+        <x:v>13133.4052</x:v>
+      </x:c>
+      <x:c r="C213" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="28" customHeight="1">
+      <x:c r="A214" s="18" t="str">
+        <x:v>known_required_high_TWD</x:v>
+      </x:c>
+      <x:c r="B214" s="18" t="str">
+        <x:v>13133.4052</x:v>
+      </x:c>
+      <x:c r="C214" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="28" customHeight="1">
+      <x:c r="A215" s="18" t="str">
+        <x:v>known_nonPCB_low_TWD</x:v>
+      </x:c>
+      <x:c r="B215" s="18" t="str">
+        <x:v>14248.790799999999</x:v>
+      </x:c>
+      <x:c r="C215" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="28" customHeight="1">
+      <x:c r="A216" s="18" t="str">
+        <x:v>known_nonPCB_high_TWD</x:v>
+      </x:c>
+      <x:c r="B216" s="18" t="str">
+        <x:v>14248.790799999999</x:v>
+      </x:c>
+      <x:c r="C216" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" ht="28" customHeight="1">
+      <x:c r="A217" s="18" t="str">
+        <x:v>known_partial_low_TWD</x:v>
+      </x:c>
+      <x:c r="B217" s="18" t="str">
+        <x:v>79873.7908</x:v>
+      </x:c>
+      <x:c r="C217" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218" ht="28" customHeight="1">
+      <x:c r="A218" s="18" t="str">
+        <x:v>known_partial_high_TWD</x:v>
+      </x:c>
+      <x:c r="B218" s="18" t="str">
+        <x:v>79873.7908</x:v>
+      </x:c>
+      <x:c r="C218" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="28" customHeight="1">
+      <x:c r="A219" s="18" t="str">
+        <x:v>required_budget_NTD</x:v>
+      </x:c>
+      <x:c r="B219" s="18" t="str">
+        <x:v>79873.7908</x:v>
+      </x:c>
+      <x:c r="C219" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" ht="28" customHeight="1">
+      <x:c r="A220" s="18" t="str">
+        <x:v>required_budget_USD</x:v>
+      </x:c>
+      <x:c r="B220" s="18" t="str">
+        <x:v>2511.359559817639</x:v>
+      </x:c>
+      <x:c r="C220" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="28" customHeight="1">
+      <x:c r="A221" s="18" t="str">
+        <x:v>required_new_packs_NTD</x:v>
+      </x:c>
+      <x:c r="B221" s="18" t="str">
+        <x:v>16300.4507</x:v>
+      </x:c>
+      <x:c r="C221" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222" ht="28" customHeight="1">
+      <x:c r="A222" s="18" t="str">
+        <x:v>developer_budget_NTD</x:v>
+      </x:c>
+      <x:c r="B222" s="18" t="str">
+        <x:v>38612.18275</x:v>
+      </x:c>
+      <x:c r="C222" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223" ht="28" customHeight="1">
+      <x:c r="A223" s="18" t="str">
+        <x:v>developer_budget_USD</x:v>
+      </x:c>
+      <x:c r="B223" s="18" t="str">
+        <x:v>1214.0286983178746</x:v>
+      </x:c>
+      <x:c r="C223" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224" ht="28" customHeight="1">
+      <x:c r="A224" s="18" t="str">
+        <x:v>future_budget_NTD</x:v>
+      </x:c>
+      <x:c r="B224" s="18" t="str">
+        <x:v>7500</x:v>
+      </x:c>
+      <x:c r="C224" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225" ht="28" customHeight="1">
+      <x:c r="A225" s="18" t="str">
+        <x:v>complete_cost</x:v>
+      </x:c>
+      <x:c r="B225" s="18" t="str">
+        <x:v>Not order-ready; proxies and allowances included</x:v>
+      </x:c>
+      <x:c r="C225" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226" ht="40" customHeight="1">
+      <x:c r="A226" s="18" t="str">
+        <x:v>formula_total_matches_inde
+pendent_calculation</x:v>
+      </x:c>
+      <x:c r="B226" s="18" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="C226" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227" ht="28" customHeight="1">
+      <x:c r="A227" s="18" t="str">
+        <x:v>blank_vs_zero_test_passed</x:v>
+      </x:c>
+      <x:c r="B227" s="18" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="C227" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228" ht="28" customHeight="1">
+      <x:c r="A228" s="18" t="str">
+        <x:v>pack_vs_usage_test_passed</x:v>
+      </x:c>
+      <x:c r="B228" s="18" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="C228" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229" ht="28" customHeight="1">
+      <x:c r="A229" s="18" t="str">
+        <x:v>owned_quantity_test_passed</x:v>
+      </x:c>
+      <x:c r="B229" s="18" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="C229" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230" ht="28" customHeight="1">
+      <x:c r="A230" s="18" t="str">
+        <x:v>FX_recalculation_passed</x:v>
+      </x:c>
+      <x:c r="B230" s="18" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="C230" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231" ht="28" customHeight="1">
+      <x:c r="A231" s="18" t="str">
+        <x:v>zero_FX_rejected</x:v>
+      </x:c>
+      <x:c r="B231" s="18" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="C231" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232" ht="28" customHeight="1">
+      <x:c r="A232" s="18" t="str">
+        <x:v>zero_PCB_divisor_rejected</x:v>
+      </x:c>
+      <x:c r="B232" s="18" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="C232" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233" ht="40" customHeight="1">
+      <x:c r="A233" s="18" t="str">
+        <x:v>source_total_excluded_from
+_costs</x:v>
+      </x:c>
+      <x:c r="B233" s="18" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="C233" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234" ht="28" customHeight="1">
+      <x:c r="A234" s="18" t="str">
+        <x:v>public_workbook_updated</x:v>
+      </x:c>
+      <x:c r="B234" s="18" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="C234" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235" ht="28" customHeight="1">
+      <x:c r="A235" s="18" t="str">
+        <x:v>public_workbook_sha256</x:v>
+      </x:c>
+      <x:c r="B235" s="18" t="str">
+        <x:v>46de0bf3fb0d699ceeccc2e301d47868e6a5fb8ea916e7a284ff12288f4c707e</x:v>
+      </x:c>
+      <x:c r="C235" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236" ht="28" customHeight="1">
+      <x:c r="A236" s="18" t="str">
+        <x:v>staged_workbook_sha256</x:v>
+      </x:c>
+      <x:c r="B236" s="18" t="str">
+        <x:v>46de0bf3fb0d699ceeccc2e301d47868e6a5fb8ea916e7a284ff12288f4c707e</x:v>
+      </x:c>
+      <x:c r="C236" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237" ht="28" customHeight="1">
+      <x:c r="A237" s="18" t="str">
+        <x:v>visual_QA_passed</x:v>
+      </x:c>
+      <x:c r="B237" s="18" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="C237" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238" ht="28" customHeight="1">
+      <x:c r="A238" s="18" t="str">
+        <x:v>rendered_sheets</x:v>
+      </x:c>
+      <x:c r="B238" s="18" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C238" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239" ht="28" customHeight="1">
+      <x:c r="A239" s="18" t="str">
+        <x:v>rendered_ranges</x:v>
+      </x:c>
+      <x:c r="B239" s="18" t="str">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C239" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240" ht="40" customHeight="1">
+      <x:c r="A240" s="18" t="str">
+        <x:v>visual_QA</x:v>
+      </x:c>
+      <x:c r="B240" s="18" t="str">
+        <x:v>All five worksheets and all 37 rendered ranges inspected, including every purchase and PCB row. Formula checks use artifact-tool; native Excel rendering is not claimed.</x:v>
+      </x:c>
+      <x:c r="C240" s="18" t="str">
+        <x:v>先前驗證紀錄。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>